<commit_message>
chore: 自動更新最新基金與ETF數據 (2026-10-19 17:13:54)
</commit_message>
<xml_diff>
--- a/國泰投信_人氣ETF與熱門基金分析.xlsx
+++ b/國泰投信_人氣ETF與熱門基金分析.xlsx
@@ -207,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -230,7 +230,7 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -239,13 +239,13 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="10" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="10" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -338,7 +338,7 @@
     <xf numFmtId="4" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -350,19 +350,31 @@
     <xf numFmtId="4" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="10" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="10" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="4" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="10" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1713,7 +1725,7 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>國泰台灣科技龍頭 (00881) (台積電佔比: 39.96% (科技純度: 95.34%))</t>
+          <t>國泰台灣科技龍頭 (00881) (台積電佔比: 39.86% (科技純度: 95.26%))</t>
         </is>
       </c>
     </row>
@@ -2946,7 +2958,7 @@
         <v>48.7</v>
       </c>
       <c r="H10" s="29" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="I10" s="31" t="n">
         <v>0</v>
@@ -6380,7 +6392,7 @@
         <v>0.09939999999999999</v>
       </c>
       <c r="H70" s="32" t="n">
-        <v/>
+        <v>42.48</v>
       </c>
       <c r="I70" s="27" t="inlineStr">
         <is>
@@ -6392,9 +6404,9 @@
           <t>2026/11/12</t>
         </is>
       </c>
-      <c r="K70" s="26" t="inlineStr">
-        <is>
-          <t>資料不足</t>
+      <c r="K70" s="33" t="inlineStr">
+        <is>
+          <t>尚未填息 (貼息中)</t>
         </is>
       </c>
       <c r="L70" s="34" t="n">
@@ -13085,22 +13097,22 @@
         </is>
       </c>
       <c r="D5" s="23" t="n">
-        <v>0.08810000000000001</v>
+        <v>0.08710000000000001</v>
       </c>
       <c r="E5" s="23" t="n">
-        <v>0.6870999999999998</v>
+        <v>0.6758999999999999</v>
       </c>
       <c r="F5" s="23" t="n">
-        <v>0.7751999999999998</v>
+        <v>0.7629999999999998</v>
       </c>
       <c r="G5" s="23" t="n">
-        <v>0.0327</v>
+        <v>0.032</v>
       </c>
       <c r="H5" s="23" t="n">
-        <v>0.1217</v>
+        <v>0.118</v>
       </c>
       <c r="I5" s="21" t="n">
-        <v>0.0086</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="J5" s="21" t="inlineStr">
         <is>
@@ -13109,7 +13121,7 @@
       </c>
       <c r="K5" s="21" t="inlineStr">
         <is>
-          <t>台積電(8.81%), 聯發科(6.29%), 台光電(4.36%)</t>
+          <t>台積電(8.71%), 聯發科(6.16%), 台光電(4.28%)</t>
         </is>
       </c>
     </row>
@@ -13265,22 +13277,22 @@
         </is>
       </c>
       <c r="D9" s="23" t="n">
-        <v>0.3996</v>
+        <v>0.3986</v>
       </c>
       <c r="E9" s="23" t="n">
-        <v>0.5538</v>
+        <v>0.5539999999999999</v>
       </c>
       <c r="F9" s="23" t="n">
-        <v>0.9534</v>
+        <v>0.9525999999999999</v>
       </c>
       <c r="G9" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="23" t="n">
-        <v>0.0247</v>
+        <v>0.0213</v>
       </c>
       <c r="I9" s="21" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="J9" s="21" t="inlineStr">
         <is>
@@ -13289,7 +13301,7 @@
       </c>
       <c r="K9" s="21" t="inlineStr">
         <is>
-          <t>台積電(39.96%), 聯發科(10.21%), 台達電(5.47%)</t>
+          <t>台積電(39.86%), 聯發科(10.08%), 台達電(5.47%)</t>
         </is>
       </c>
     </row>
@@ -13415,7 +13427,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="27" t="n">
-        <v>0.9998999999999999</v>
+        <v>0.9996999999999998</v>
       </c>
       <c r="J12" s="27" t="inlineStr">
         <is>
@@ -13424,7 +13436,7 @@
       </c>
       <c r="K12" s="27" t="inlineStr">
         <is>
-          <t>Apple Inc.(17.29%), Microsoft Corp(14.34%), AMAZON.COM INC(9.02%)</t>
+          <t>Apple Inc.(17.5%), Microsoft Corp(14.17%), AMAZON.COM INC(8.92%)</t>
         </is>
       </c>
     </row>
@@ -13490,22 +13502,22 @@
         </is>
       </c>
       <c r="D14" s="29" t="n">
-        <v>0.2264</v>
+        <v>0.2261</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.4193000000000001</v>
+        <v>0.4155</v>
       </c>
       <c r="F14" s="29" t="n">
-        <v>0.6457000000000001</v>
+        <v>0.6415999999999999</v>
       </c>
       <c r="G14" s="31" t="n">
         <v>0</v>
       </c>
       <c r="H14" s="29" t="n">
-        <v>0.0095</v>
+        <v>0.009399999999999999</v>
       </c>
       <c r="I14" s="27" t="n">
-        <v>0.3249</v>
+        <v>0.3295999999999999</v>
       </c>
       <c r="J14" s="27" t="inlineStr">
         <is>
@@ -13514,7 +13526,7 @@
       </c>
       <c r="K14" s="27" t="inlineStr">
         <is>
-          <t>台積電(22.64%), Samsung Electron Rg(14.8%), SK Hynix Inc(11.19%)</t>
+          <t>台積電(22.61%), Samsung Electron Rg(15.03%), SK Hynix Inc(11.28%)</t>
         </is>
       </c>
     </row>
@@ -13550,7 +13562,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="21" t="n">
-        <v>0.9981999999999996</v>
+        <v>0.9980999999999999</v>
       </c>
       <c r="J15" s="21" t="inlineStr">
         <is>
@@ -13559,7 +13571,7 @@
       </c>
       <c r="K15" s="21" t="inlineStr">
         <is>
-          <t>NVIDIA CORPORATION(11.77%), BROADCOM INC(9.27%), Micron Technology Inc(7.75%)</t>
+          <t>NVIDIA CORPORATION(12.07%), BROADCOM INC(9.2%), Micron Technology Inc(7.6%)</t>
         </is>
       </c>
     </row>
@@ -13595,7 +13607,7 @@
         <v>0</v>
       </c>
       <c r="I16" s="27" t="n">
-        <v>0.9856000000000023</v>
+        <v>0.9868000000000027</v>
       </c>
       <c r="J16" s="27" t="inlineStr">
         <is>
@@ -13604,7 +13616,7 @@
       </c>
       <c r="K16" s="27" t="inlineStr">
         <is>
-          <t>Microsoft Corp(9.07%), Apple Inc.(8.97%), NVIDIA CORPORATION(8.03%)</t>
+          <t>Apple Inc.(9.33%), Microsoft Corp(9.22%), NVIDIA CORPORATION(8.2%)</t>
         </is>
       </c>
     </row>
@@ -13628,10 +13640,10 @@
         <v>0</v>
       </c>
       <c r="E17" s="23" t="n">
-        <v>0.0336</v>
+        <v>0.0346</v>
       </c>
       <c r="F17" s="23" t="n">
-        <v>0.0336</v>
+        <v>0.0346</v>
       </c>
       <c r="G17" s="25" t="n">
         <v>0</v>
@@ -13640,7 +13652,7 @@
         <v>0</v>
       </c>
       <c r="I17" s="21" t="n">
-        <v>0.9536999999999998</v>
+        <v>0.9529999999999998</v>
       </c>
       <c r="J17" s="21" t="inlineStr">
         <is>
@@ -13649,7 +13661,7 @@
       </c>
       <c r="K17" s="21" t="inlineStr">
         <is>
-          <t>ADV MICRO DEVICES(26.81%), NVIDIA CORPORATION(14.26%), TESLA, INC.(11.98%)</t>
+          <t>ADV MICRO DEVICES(25.83%), NVIDIA CORPORATION(14.41%), TESLA, INC.(12.01%)</t>
         </is>
       </c>
     </row>
@@ -14237,7 +14249,7 @@
         </is>
       </c>
       <c r="H33" s="23" t="n">
-        <v>0.08810000000000001</v>
+        <v>0.08710000000000001</v>
       </c>
       <c r="I33" s="21" t="inlineStr">
         <is>
@@ -14280,7 +14292,7 @@
         </is>
       </c>
       <c r="H34" s="29" t="n">
-        <v>0.0629</v>
+        <v>0.0616</v>
       </c>
       <c r="I34" s="27" t="inlineStr">
         <is>
@@ -14323,7 +14335,7 @@
         </is>
       </c>
       <c r="H35" s="25" t="n">
-        <v>0.0436</v>
+        <v>0.0428</v>
       </c>
       <c r="I35" s="21" t="inlineStr">
         <is>
@@ -14366,7 +14378,7 @@
         </is>
       </c>
       <c r="H36" s="31" t="n">
-        <v>0.0426</v>
+        <v>0.0416</v>
       </c>
       <c r="I36" s="27" t="inlineStr">
         <is>
@@ -14409,7 +14421,7 @@
         </is>
       </c>
       <c r="H37" s="25" t="n">
-        <v>0.0388</v>
+        <v>0.0394</v>
       </c>
       <c r="I37" s="21" t="inlineStr">
         <is>
@@ -14452,7 +14464,7 @@
         </is>
       </c>
       <c r="H38" s="31" t="n">
-        <v>0.0363</v>
+        <v>0.0359</v>
       </c>
       <c r="I38" s="27" t="inlineStr">
         <is>
@@ -14495,7 +14507,7 @@
         </is>
       </c>
       <c r="H39" s="25" t="n">
-        <v>0.0345</v>
+        <v>0.0332</v>
       </c>
       <c r="I39" s="21" t="inlineStr">
         <is>
@@ -14538,7 +14550,7 @@
         </is>
       </c>
       <c r="H40" s="31" t="n">
-        <v>0.0313</v>
+        <v>0.0312</v>
       </c>
       <c r="I40" s="27" t="inlineStr">
         <is>
@@ -14581,7 +14593,7 @@
         </is>
       </c>
       <c r="H41" s="25" t="n">
-        <v>0.0313</v>
+        <v>0.031</v>
       </c>
       <c r="I41" s="21" t="inlineStr">
         <is>
@@ -14610,25 +14622,25 @@
       </c>
       <c r="E42" s="26" t="inlineStr">
         <is>
-          <t>2059</t>
+          <t>2368</t>
         </is>
       </c>
       <c r="F42" s="27" t="inlineStr">
         <is>
-          <t>川湖</t>
+          <t>金像電</t>
         </is>
       </c>
       <c r="G42" s="27" t="inlineStr">
         <is>
-          <t>傳統產業</t>
+          <t>科技電子</t>
         </is>
       </c>
       <c r="H42" s="31" t="n">
-        <v>0.0305</v>
+        <v>0.0302</v>
       </c>
       <c r="I42" s="27" t="inlineStr">
         <is>
-          <t>92,000</t>
+          <t>734,000</t>
         </is>
       </c>
     </row>
@@ -15797,7 +15809,7 @@
         </is>
       </c>
       <c r="H73" s="23" t="n">
-        <v>0.3996</v>
+        <v>0.3986</v>
       </c>
       <c r="I73" s="21" t="inlineStr">
         <is>
@@ -15840,7 +15852,7 @@
         </is>
       </c>
       <c r="H74" s="29" t="n">
-        <v>0.1021</v>
+        <v>0.1008</v>
       </c>
       <c r="I74" s="27" t="inlineStr">
         <is>
@@ -15926,7 +15938,7 @@
         </is>
       </c>
       <c r="H76" s="31" t="n">
-        <v>0.0471</v>
+        <v>0.0461</v>
       </c>
       <c r="I76" s="27" t="inlineStr">
         <is>
@@ -15969,11 +15981,11 @@
         </is>
       </c>
       <c r="H77" s="25" t="n">
-        <v>0.0303</v>
+        <v>0.0292</v>
       </c>
       <c r="I77" s="21" t="inlineStr">
         <is>
-          <t>4,122,871</t>
+          <t>3,872,871</t>
         </is>
       </c>
     </row>
@@ -16012,11 +16024,11 @@
         </is>
       </c>
       <c r="H78" s="31" t="n">
-        <v>0.0288</v>
+        <v>0.0265</v>
       </c>
       <c r="I78" s="27" t="inlineStr">
         <is>
-          <t>32,111,000</t>
+          <t>29,935,000</t>
         </is>
       </c>
     </row>
@@ -16055,7 +16067,7 @@
         </is>
       </c>
       <c r="H79" s="25" t="n">
-        <v>0.0267</v>
+        <v>0.0265</v>
       </c>
       <c r="I79" s="21" t="inlineStr">
         <is>
@@ -16127,25 +16139,25 @@
       </c>
       <c r="E81" s="20" t="inlineStr">
         <is>
-          <t>2059</t>
+          <t>2345</t>
         </is>
       </c>
       <c r="F81" s="21" t="inlineStr">
         <is>
-          <t>川湖</t>
+          <t>智邦</t>
         </is>
       </c>
       <c r="G81" s="21" t="inlineStr">
         <is>
-          <t>傳統產業</t>
+          <t>科技電子</t>
         </is>
       </c>
       <c r="H81" s="25" t="n">
-        <v>0.0227</v>
+        <v>0.0224</v>
       </c>
       <c r="I81" s="21" t="inlineStr">
         <is>
-          <t>338,000</t>
+          <t>1,663,000</t>
         </is>
       </c>
     </row>
@@ -16170,25 +16182,25 @@
       </c>
       <c r="E82" s="26" t="inlineStr">
         <is>
-          <t>2345</t>
+          <t>2059</t>
         </is>
       </c>
       <c r="F82" s="27" t="inlineStr">
         <is>
-          <t>智邦</t>
+          <t>川湖</t>
         </is>
       </c>
       <c r="G82" s="27" t="inlineStr">
         <is>
-          <t>科技電子</t>
+          <t>傳統產業</t>
         </is>
       </c>
       <c r="H82" s="31" t="n">
-        <v>0.0222</v>
+        <v>0.021</v>
       </c>
       <c r="I82" s="27" t="inlineStr">
         <is>
-          <t>1,663,000</t>
+          <t>315,000</t>
         </is>
       </c>
     </row>
@@ -16657,11 +16669,11 @@
         </is>
       </c>
       <c r="H93" s="23" t="n">
-        <v>0.1729</v>
+        <v>0.175</v>
       </c>
       <c r="I93" s="21" t="inlineStr">
         <is>
-          <t>40,391</t>
+          <t>40,189</t>
         </is>
       </c>
     </row>
@@ -16700,11 +16712,11 @@
         </is>
       </c>
       <c r="H94" s="29" t="n">
-        <v>0.1434</v>
+        <v>0.1417</v>
       </c>
       <c r="I94" s="27" t="inlineStr">
         <is>
-          <t>21,241</t>
+          <t>21,135</t>
         </is>
       </c>
     </row>
@@ -16743,11 +16755,11 @@
         </is>
       </c>
       <c r="H95" s="23" t="n">
-        <v>0.0902</v>
+        <v>0.0892</v>
       </c>
       <c r="I95" s="21" t="inlineStr">
         <is>
-          <t>28,294</t>
+          <t>28,146</t>
         </is>
       </c>
     </row>
@@ -16786,11 +16798,11 @@
         </is>
       </c>
       <c r="H96" s="29" t="n">
-        <v>0.0738</v>
+        <v>0.0725</v>
       </c>
       <c r="I96" s="27" t="inlineStr">
         <is>
-          <t>16,875</t>
+          <t>16,787</t>
         </is>
       </c>
     </row>
@@ -16829,11 +16841,11 @@
         </is>
       </c>
       <c r="H97" s="23" t="n">
-        <v>0.05860000000000001</v>
+        <v>0.0568</v>
       </c>
       <c r="I97" s="21" t="inlineStr">
         <is>
-          <t>6,353</t>
+          <t>6,320</t>
         </is>
       </c>
     </row>
@@ -16872,11 +16884,11 @@
         </is>
       </c>
       <c r="H98" s="31" t="n">
-        <v>0.0372</v>
+        <v>0.0366</v>
       </c>
       <c r="I98" s="27" t="inlineStr">
         <is>
-          <t>8,189</t>
+          <t>8,146</t>
         </is>
       </c>
     </row>
@@ -16915,11 +16927,11 @@
         </is>
       </c>
       <c r="H99" s="25" t="n">
-        <v>0.0328</v>
+        <v>0.0335</v>
       </c>
       <c r="I99" s="21" t="inlineStr">
         <is>
-          <t>7,809</t>
+          <t>7,768</t>
         </is>
       </c>
     </row>
@@ -16958,11 +16970,11 @@
         </is>
       </c>
       <c r="H100" s="31" t="n">
-        <v>0.0285</v>
+        <v>0.0295</v>
       </c>
       <c r="I100" s="27" t="inlineStr">
         <is>
-          <t>14,582</t>
+          <t>14,408</t>
         </is>
       </c>
     </row>
@@ -17001,11 +17013,11 @@
         </is>
       </c>
       <c r="H101" s="25" t="n">
-        <v>0.0244</v>
+        <v>0.0248</v>
       </c>
       <c r="I101" s="21" t="inlineStr">
         <is>
-          <t>4,878</t>
+          <t>4,853</t>
         </is>
       </c>
     </row>
@@ -17044,11 +17056,11 @@
         </is>
       </c>
       <c r="H102" s="31" t="n">
-        <v>0.0188</v>
+        <v>0.0191</v>
       </c>
       <c r="I102" s="27" t="inlineStr">
         <is>
-          <t>12,724</t>
+          <t>12,657</t>
         </is>
       </c>
     </row>
@@ -17517,7 +17529,7 @@
         </is>
       </c>
       <c r="H113" s="23" t="n">
-        <v>0.2264</v>
+        <v>0.2261</v>
       </c>
       <c r="I113" s="21" t="inlineStr">
         <is>
@@ -17560,7 +17572,7 @@
         </is>
       </c>
       <c r="H114" s="29" t="n">
-        <v>0.148</v>
+        <v>0.1503</v>
       </c>
       <c r="I114" s="27" t="inlineStr">
         <is>
@@ -17603,7 +17615,7 @@
         </is>
       </c>
       <c r="H115" s="23" t="n">
-        <v>0.1119</v>
+        <v>0.1128</v>
       </c>
       <c r="I115" s="21" t="inlineStr">
         <is>
@@ -17646,7 +17658,7 @@
         </is>
       </c>
       <c r="H116" s="31" t="n">
-        <v>0.04219999999999999</v>
+        <v>0.0417</v>
       </c>
       <c r="I116" s="27" t="inlineStr">
         <is>
@@ -17689,7 +17701,7 @@
         </is>
       </c>
       <c r="H117" s="25" t="n">
-        <v>0.0302</v>
+        <v>0.0301</v>
       </c>
       <c r="I117" s="21" t="inlineStr">
         <is>
@@ -17732,7 +17744,7 @@
         </is>
       </c>
       <c r="H118" s="31" t="n">
-        <v>0.0247</v>
+        <v>0.0242</v>
       </c>
       <c r="I118" s="27" t="inlineStr">
         <is>
@@ -17775,7 +17787,7 @@
         </is>
       </c>
       <c r="H119" s="25" t="n">
-        <v>0.0219</v>
+        <v>0.0217</v>
       </c>
       <c r="I119" s="21" t="inlineStr">
         <is>
@@ -17804,12 +17816,12 @@
       </c>
       <c r="E120" s="26" t="inlineStr">
         <is>
-          <t>2303</t>
+          <t>3037</t>
         </is>
       </c>
       <c r="F120" s="27" t="inlineStr">
         <is>
-          <t>聯電</t>
+          <t>欣興</t>
         </is>
       </c>
       <c r="G120" s="27" t="inlineStr">
@@ -17822,7 +17834,7 @@
       </c>
       <c r="I120" s="27" t="inlineStr">
         <is>
-          <t>1,620,000</t>
+          <t>193,315</t>
         </is>
       </c>
     </row>
@@ -17847,12 +17859,12 @@
       </c>
       <c r="E121" s="20" t="inlineStr">
         <is>
-          <t>3037</t>
+          <t>2303</t>
         </is>
       </c>
       <c r="F121" s="21" t="inlineStr">
         <is>
-          <t>欣興</t>
+          <t>聯電</t>
         </is>
       </c>
       <c r="G121" s="21" t="inlineStr">
@@ -17861,11 +17873,11 @@
         </is>
       </c>
       <c r="H121" s="25" t="n">
-        <v>0.0201</v>
+        <v>0.0203</v>
       </c>
       <c r="I121" s="21" t="inlineStr">
         <is>
-          <t>193,315</t>
+          <t>1,620,000</t>
         </is>
       </c>
     </row>
@@ -17947,11 +17959,11 @@
         </is>
       </c>
       <c r="H123" s="23" t="n">
-        <v>0.1177</v>
+        <v>0.1207</v>
       </c>
       <c r="I123" s="21" t="inlineStr">
         <is>
-          <t>1,246,077</t>
+          <t>1,270,494</t>
         </is>
       </c>
     </row>
@@ -17990,11 +18002,11 @@
         </is>
       </c>
       <c r="H124" s="29" t="n">
-        <v>0.09269999999999999</v>
+        <v>0.092</v>
       </c>
       <c r="I124" s="27" t="inlineStr">
         <is>
-          <t>619,070</t>
+          <t>631,201</t>
         </is>
       </c>
     </row>
@@ -18033,11 +18045,11 @@
         </is>
       </c>
       <c r="H125" s="23" t="n">
-        <v>0.0775</v>
+        <v>0.076</v>
       </c>
       <c r="I125" s="21" t="inlineStr">
         <is>
-          <t>191,309</t>
+          <t>195,057</t>
         </is>
       </c>
     </row>
@@ -18076,11 +18088,11 @@
         </is>
       </c>
       <c r="H126" s="31" t="n">
-        <v>0.0476</v>
+        <v>0.0466</v>
       </c>
       <c r="I126" s="27" t="inlineStr">
         <is>
-          <t>194,822</t>
+          <t>198,639</t>
         </is>
       </c>
     </row>
@@ -18105,12 +18117,12 @@
       </c>
       <c r="E127" s="20" t="inlineStr">
         <is>
-          <t>MRVL.US</t>
+          <t>ADI.US</t>
         </is>
       </c>
       <c r="F127" s="21" t="inlineStr">
         <is>
-          <t>MARVELL TECH GROUP</t>
+          <t>ANALOG DEVICES INC</t>
         </is>
       </c>
       <c r="G127" s="21" t="inlineStr">
@@ -18119,11 +18131,11 @@
         </is>
       </c>
       <c r="H127" s="25" t="n">
-        <v>0.0455</v>
+        <v>0.0453</v>
       </c>
       <c r="I127" s="21" t="inlineStr">
         <is>
-          <t>433,273</t>
+          <t>258,197</t>
         </is>
       </c>
     </row>
@@ -18148,12 +18160,12 @@
       </c>
       <c r="E128" s="26" t="inlineStr">
         <is>
-          <t>ADI.US</t>
+          <t>MRVL.US</t>
         </is>
       </c>
       <c r="F128" s="27" t="inlineStr">
         <is>
-          <t>ANALOG DEVICES INC</t>
+          <t>MARVELL TECH GROUP</t>
         </is>
       </c>
       <c r="G128" s="27" t="inlineStr">
@@ -18162,11 +18174,11 @@
         </is>
       </c>
       <c r="H128" s="31" t="n">
-        <v>0.0445</v>
+        <v>0.0446</v>
       </c>
       <c r="I128" s="27" t="inlineStr">
         <is>
-          <t>253,235</t>
+          <t>441,763</t>
         </is>
       </c>
     </row>
@@ -18205,11 +18217,11 @@
         </is>
       </c>
       <c r="H129" s="25" t="n">
-        <v>0.04269999999999999</v>
+        <v>0.04389999999999999</v>
       </c>
       <c r="I129" s="21" t="inlineStr">
         <is>
-          <t>351,488</t>
+          <t>358,375</t>
         </is>
       </c>
     </row>
@@ -18234,12 +18246,12 @@
       </c>
       <c r="E130" s="26" t="inlineStr">
         <is>
-          <t>INTC.US</t>
+          <t>QCOM.US</t>
         </is>
       </c>
       <c r="F130" s="27" t="inlineStr">
         <is>
-          <t>Intel Corp</t>
+          <t>QUALCOMM INC</t>
         </is>
       </c>
       <c r="G130" s="27" t="inlineStr">
@@ -18248,11 +18260,11 @@
         </is>
       </c>
       <c r="H130" s="31" t="n">
-        <v>0.0425</v>
+        <v>0.04190000000000001</v>
       </c>
       <c r="I130" s="27" t="inlineStr">
         <is>
-          <t>1,024,540</t>
+          <t>548,472</t>
         </is>
       </c>
     </row>
@@ -18277,12 +18289,12 @@
       </c>
       <c r="E131" s="20" t="inlineStr">
         <is>
-          <t>QCOM.US</t>
+          <t>INTC.US</t>
         </is>
       </c>
       <c r="F131" s="21" t="inlineStr">
         <is>
-          <t>QUALCOMM INC</t>
+          <t>Intel Corp</t>
         </is>
       </c>
       <c r="G131" s="21" t="inlineStr">
@@ -18291,11 +18303,11 @@
         </is>
       </c>
       <c r="H131" s="25" t="n">
-        <v>0.0417</v>
+        <v>0.0416</v>
       </c>
       <c r="I131" s="21" t="inlineStr">
         <is>
-          <t>537,932</t>
+          <t>1,044,616</t>
         </is>
       </c>
     </row>
@@ -18334,11 +18346,11 @@
         </is>
       </c>
       <c r="H132" s="31" t="n">
-        <v>0.0405</v>
+        <v>0.0412</v>
       </c>
       <c r="I132" s="27" t="inlineStr">
         <is>
-          <t>220,810</t>
+          <t>225,136</t>
         </is>
       </c>
     </row>
@@ -18363,12 +18375,12 @@
       </c>
       <c r="E133" s="20" t="inlineStr">
         <is>
-          <t>MSFT.US</t>
+          <t>AAPL.US</t>
         </is>
       </c>
       <c r="F133" s="21" t="inlineStr">
         <is>
-          <t>Microsoft Corp</t>
+          <t>Apple Inc.</t>
         </is>
       </c>
       <c r="G133" s="21" t="inlineStr">
@@ -18377,11 +18389,11 @@
         </is>
       </c>
       <c r="H133" s="23" t="n">
-        <v>0.0907</v>
+        <v>0.09329999999999999</v>
       </c>
       <c r="I133" s="21" t="inlineStr">
         <is>
-          <t>31,412</t>
+          <t>50,314</t>
         </is>
       </c>
     </row>
@@ -18406,12 +18418,12 @@
       </c>
       <c r="E134" s="26" t="inlineStr">
         <is>
-          <t>AAPL.US</t>
+          <t>MSFT.US</t>
         </is>
       </c>
       <c r="F134" s="27" t="inlineStr">
         <is>
-          <t>Apple Inc.</t>
+          <t>Microsoft Corp</t>
         </is>
       </c>
       <c r="G134" s="27" t="inlineStr">
@@ -18420,11 +18432,11 @@
         </is>
       </c>
       <c r="H134" s="29" t="n">
-        <v>0.0897</v>
+        <v>0.0922</v>
       </c>
       <c r="I134" s="27" t="inlineStr">
         <is>
-          <t>48,975</t>
+          <t>32,271</t>
         </is>
       </c>
     </row>
@@ -18463,11 +18475,11 @@
         </is>
       </c>
       <c r="H135" s="23" t="n">
-        <v>0.0803</v>
+        <v>0.08199999999999999</v>
       </c>
       <c r="I135" s="21" t="inlineStr">
         <is>
-          <t>69,047</t>
+          <t>70,935</t>
         </is>
       </c>
     </row>
@@ -18506,11 +18518,11 @@
         </is>
       </c>
       <c r="H136" s="29" t="n">
-        <v>0.0706</v>
+        <v>0.0698</v>
       </c>
       <c r="I136" s="27" t="inlineStr">
         <is>
-          <t>38,297</t>
+          <t>39,344</t>
         </is>
       </c>
     </row>
@@ -18549,11 +18561,11 @@
         </is>
       </c>
       <c r="H137" s="25" t="n">
-        <v>0.0493</v>
+        <v>0.0492</v>
       </c>
       <c r="I137" s="21" t="inlineStr">
         <is>
-          <t>12,508</t>
+          <t>12,850</t>
         </is>
       </c>
     </row>
@@ -18592,11 +18604,11 @@
         </is>
       </c>
       <c r="H138" s="31" t="n">
-        <v>0.0484</v>
+        <v>0.0489</v>
       </c>
       <c r="I138" s="27" t="inlineStr">
         <is>
-          <t>25,884</t>
+          <t>26,592</t>
         </is>
       </c>
     </row>
@@ -18635,11 +18647,11 @@
         </is>
       </c>
       <c r="H139" s="25" t="n">
-        <v>0.0417</v>
+        <v>0.0406</v>
       </c>
       <c r="I139" s="21" t="inlineStr">
         <is>
-          <t>13,851</t>
+          <t>14,230</t>
         </is>
       </c>
     </row>
@@ -18664,12 +18676,12 @@
       </c>
       <c r="E140" s="26" t="inlineStr">
         <is>
-          <t>MU.US</t>
+          <t>GOOG.US</t>
         </is>
       </c>
       <c r="F140" s="27" t="inlineStr">
         <is>
-          <t>Micron Technology Inc</t>
+          <t>ALPHABET INC-CL C</t>
         </is>
       </c>
       <c r="G140" s="27" t="inlineStr">
@@ -18678,11 +18690,11 @@
         </is>
       </c>
       <c r="H140" s="31" t="n">
-        <v>0.0397</v>
+        <v>0.0392</v>
       </c>
       <c r="I140" s="27" t="inlineStr">
         <is>
-          <t>7,955</t>
+          <t>21,540</t>
         </is>
       </c>
     </row>
@@ -18707,12 +18719,12 @@
       </c>
       <c r="E141" s="20" t="inlineStr">
         <is>
-          <t>GOOG.US</t>
+          <t>MU.US</t>
         </is>
       </c>
       <c r="F141" s="21" t="inlineStr">
         <is>
-          <t>ALPHABET INC-CL C</t>
+          <t>Micron Technology Inc</t>
         </is>
       </c>
       <c r="G141" s="21" t="inlineStr">
@@ -18721,11 +18733,11 @@
         </is>
       </c>
       <c r="H141" s="25" t="n">
-        <v>0.0387</v>
+        <v>0.0388</v>
       </c>
       <c r="I141" s="21" t="inlineStr">
         <is>
-          <t>20,967</t>
+          <t>8,173</t>
         </is>
       </c>
     </row>
@@ -18764,11 +18776,11 @@
         </is>
       </c>
       <c r="H142" s="31" t="n">
-        <v>0.0215</v>
+        <v>0.021</v>
       </c>
       <c r="I142" s="27" t="inlineStr">
         <is>
-          <t>42,161</t>
+          <t>43,313</t>
         </is>
       </c>
     </row>
@@ -18807,7 +18819,7 @@
         </is>
       </c>
       <c r="H143" s="23" t="n">
-        <v>0.2681</v>
+        <v>0.2583</v>
       </c>
       <c r="I143" s="21" t="inlineStr">
         <is>
@@ -18850,7 +18862,7 @@
         </is>
       </c>
       <c r="H144" s="29" t="n">
-        <v>0.1426</v>
+        <v>0.1441</v>
       </c>
       <c r="I144" s="27" t="inlineStr">
         <is>
@@ -18893,7 +18905,7 @@
         </is>
       </c>
       <c r="H145" s="23" t="n">
-        <v>0.1198</v>
+        <v>0.1201</v>
       </c>
       <c r="I145" s="21" t="inlineStr">
         <is>
@@ -18936,7 +18948,7 @@
         </is>
       </c>
       <c r="H146" s="29" t="n">
-        <v>0.1015</v>
+        <v>0.103</v>
       </c>
       <c r="I146" s="27" t="inlineStr">
         <is>
@@ -18979,7 +18991,7 @@
         </is>
       </c>
       <c r="H147" s="23" t="n">
-        <v>0.0548</v>
+        <v>0.0561</v>
       </c>
       <c r="I147" s="21" t="inlineStr">
         <is>
@@ -19022,7 +19034,7 @@
         </is>
       </c>
       <c r="H148" s="31" t="n">
-        <v>0.0411</v>
+        <v>0.042</v>
       </c>
       <c r="I148" s="27" t="inlineStr">
         <is>
@@ -19065,7 +19077,7 @@
         </is>
       </c>
       <c r="H149" s="25" t="n">
-        <v>0.0375</v>
+        <v>0.0382</v>
       </c>
       <c r="I149" s="21" t="inlineStr">
         <is>
@@ -19108,7 +19120,7 @@
         </is>
       </c>
       <c r="H150" s="31" t="n">
-        <v>0.0336</v>
+        <v>0.0346</v>
       </c>
       <c r="I150" s="27" t="inlineStr">
         <is>
@@ -19151,7 +19163,7 @@
         </is>
       </c>
       <c r="H151" s="25" t="n">
-        <v>0.0272</v>
+        <v>0.0271</v>
       </c>
       <c r="I151" s="21" t="inlineStr">
         <is>
@@ -19194,7 +19206,7 @@
         </is>
       </c>
       <c r="H152" s="31" t="n">
-        <v>0.0247</v>
+        <v>0.0252</v>
       </c>
       <c r="I152" s="27" t="inlineStr">
         <is>
@@ -23627,7 +23639,7 @@
         </is>
       </c>
       <c r="F2" s="43" t="n">
-        <v>107.6</v>
+        <v>100.6</v>
       </c>
       <c r="G2" s="44" t="n">
         <v>0.00911528</v>
@@ -23685,7 +23697,7 @@
         </is>
       </c>
       <c r="F3" s="47" t="n">
-        <v>98.45</v>
+        <v>108.3</v>
       </c>
       <c r="G3" s="48" t="n">
         <v>-0.04014465</v>
@@ -23743,7 +23755,7 @@
         </is>
       </c>
       <c r="F4" s="43" t="n">
-        <v>116.02</v>
+        <v>115.17</v>
       </c>
       <c r="G4" s="44" t="n">
         <v>0.00866128</v>
@@ -23801,7 +23813,7 @@
         </is>
       </c>
       <c r="F5" s="47" t="n">
-        <v>85.62</v>
+        <v>84.95999999999999</v>
       </c>
       <c r="G5" s="49" t="n">
         <v>0.06664248</v>
@@ -23859,7 +23871,7 @@
         </is>
       </c>
       <c r="F6" s="43" t="n">
-        <v>56.66</v>
+        <v>56.22</v>
       </c>
       <c r="G6" s="44" t="n">
         <v>0.06641135000000001</v>
@@ -23917,7 +23929,7 @@
         </is>
       </c>
       <c r="F7" s="47" t="n">
-        <v>352.98</v>
+        <v>350.57</v>
       </c>
       <c r="G7" s="49" t="n">
         <v>0.04333726</v>
@@ -23975,7 +23987,7 @@
         </is>
       </c>
       <c r="F8" s="43" t="n">
-        <v>50</v>
+        <v>53.15</v>
       </c>
       <c r="G8" s="44" t="n">
         <v>0.04219119</v>
@@ -24033,7 +24045,7 @@
         </is>
       </c>
       <c r="F9" s="47" t="n">
-        <v>83.95</v>
+        <v>87.5</v>
       </c>
       <c r="G9" s="48" t="n">
         <v>-0.11655405</v>
@@ -24091,7 +24103,7 @@
         </is>
       </c>
       <c r="F10" s="43" t="n">
-        <v>175.58</v>
+        <v>174.47</v>
       </c>
       <c r="G10" s="50" t="n">
         <v>-0.04380673</v>
@@ -24149,7 +24161,7 @@
         </is>
       </c>
       <c r="F11" s="47" t="n">
-        <v>42.48</v>
+        <v>38.33</v>
       </c>
       <c r="G11" s="49" t="n">
         <v>0.05804878</v>
@@ -24207,7 +24219,7 @@
         </is>
       </c>
       <c r="F12" s="43" t="n">
-        <v>35.53</v>
+        <v>30</v>
       </c>
       <c r="G12" s="44" t="n">
         <v>0.07029505</v>
@@ -24265,7 +24277,7 @@
         </is>
       </c>
       <c r="F13" s="47" t="n">
-        <v>44.35</v>
+        <v>46.6</v>
       </c>
       <c r="G13" s="48" t="n">
         <v>-0.04295893000000001</v>
@@ -24323,7 +24335,7 @@
         </is>
       </c>
       <c r="F14" s="43" t="n">
-        <v>64.95</v>
+        <v>66.2</v>
       </c>
       <c r="G14" s="44" t="n">
         <v>0.03063547</v>
@@ -24381,7 +24393,7 @@
         </is>
       </c>
       <c r="F15" s="47" t="n">
-        <v>27.97</v>
+        <v>28.02</v>
       </c>
       <c r="G15" s="49" t="n">
         <v>0.05632139</v>
@@ -24439,7 +24451,7 @@
         </is>
       </c>
       <c r="F16" s="43" t="n">
-        <v>9.8651</v>
+        <v>9.780799999999999</v>
       </c>
       <c r="G16" s="50" t="n">
         <v>-0.02358716</v>
@@ -24497,7 +24509,7 @@
         </is>
       </c>
       <c r="F17" s="47" t="n">
-        <v>9.875299999999999</v>
+        <v>9.790900000000001</v>
       </c>
       <c r="G17" s="48" t="n">
         <v>-0.02359118</v>
@@ -24555,7 +24567,7 @@
         </is>
       </c>
       <c r="F18" s="43" t="n">
-        <v>25.82</v>
+        <v>28.56</v>
       </c>
       <c r="G18" s="50" t="n">
         <v>-0.09624573</v>
@@ -24613,7 +24625,7 @@
         </is>
       </c>
       <c r="F19" s="47" t="n">
-        <v>7.9185</v>
+        <v>7.9194</v>
       </c>
       <c r="G19" s="48" t="n">
         <v>-0.01325601</v>
@@ -24671,7 +24683,7 @@
         </is>
       </c>
       <c r="F20" s="43" t="n">
-        <v>7.8916</v>
+        <v>7.8925</v>
       </c>
       <c r="G20" s="50" t="n">
         <v>-0.01326918</v>
@@ -24729,7 +24741,7 @@
         </is>
       </c>
       <c r="F21" s="47" t="n">
-        <v>8.450900000000001</v>
+        <v>8.444000000000001</v>
       </c>
       <c r="G21" s="48" t="n">
         <v>-0.04286634</v>
@@ -24787,7 +24799,7 @@
         </is>
       </c>
       <c r="F22" s="43" t="n">
-        <v>8.448600000000001</v>
+        <v>8.441599999999999</v>
       </c>
       <c r="G22" s="50" t="n">
         <v>-0.04286672</v>
@@ -24845,7 +24857,7 @@
         </is>
       </c>
       <c r="F23" s="47" t="n">
-        <v>15.48</v>
+        <v>15.88</v>
       </c>
       <c r="G23" s="48" t="n">
         <v>-0.07210569999999999</v>
@@ -24903,7 +24915,7 @@
         </is>
       </c>
       <c r="F24" s="43" t="n">
-        <v>34.05</v>
+        <v>34.86</v>
       </c>
       <c r="G24" s="50" t="n">
         <v>-0.07485287</v>
@@ -24961,7 +24973,7 @@
         </is>
       </c>
       <c r="F25" s="47" t="n">
-        <v>15.01</v>
+        <v>14.4</v>
       </c>
       <c r="G25" s="51" t="inlineStr"/>
       <c r="H25" s="51" t="inlineStr"/>
@@ -25134,25 +25146,25 @@
         </is>
       </c>
       <c r="F2" s="43" t="n">
-        <v>15.01</v>
+        <v>14.4</v>
       </c>
       <c r="G2" s="41" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H2" s="43" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="I2" s="44" t="n">
-        <v>0.004699999999999999</v>
-      </c>
-      <c r="J2" s="52" t="inlineStr"/>
-      <c r="K2" s="52" t="inlineStr"/>
-      <c r="L2" s="52" t="inlineStr"/>
-      <c r="M2" s="52" t="inlineStr"/>
-      <c r="N2" s="52" t="inlineStr"/>
-      <c r="O2" s="52" t="inlineStr"/>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H2" s="52" t="n">
+        <v>-0.61</v>
+      </c>
+      <c r="I2" s="50" t="n">
+        <v>-0.0406</v>
+      </c>
+      <c r="J2" s="53" t="inlineStr"/>
+      <c r="K2" s="53" t="inlineStr"/>
+      <c r="L2" s="53" t="inlineStr"/>
+      <c r="M2" s="53" t="inlineStr"/>
+      <c r="N2" s="53" t="inlineStr"/>
+      <c r="O2" s="53" t="inlineStr"/>
       <c r="P2" s="41" t="inlineStr">
         <is>
           <t>月配</t>
@@ -25196,18 +25208,18 @@
         </is>
       </c>
       <c r="F3" s="47" t="n">
-        <v>35.53</v>
+        <v>30</v>
       </c>
       <c r="G3" s="45" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H3" s="47" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="I3" s="49" t="n">
-        <v>0.0125</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H3" s="54" t="n">
+        <v>-5.53</v>
+      </c>
+      <c r="I3" s="48" t="n">
+        <v>-0.1556</v>
       </c>
       <c r="J3" s="49" t="n">
         <v>0.07029505</v>
@@ -25270,18 +25282,18 @@
         </is>
       </c>
       <c r="F4" s="43" t="n">
-        <v>15.48</v>
+        <v>15.88</v>
       </c>
       <c r="G4" s="41" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H4" s="43" t="n">
-        <v>0.12</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H4" s="55" t="n">
+        <v>0.4</v>
       </c>
       <c r="I4" s="44" t="n">
-        <v>0.007800000000000001</v>
+        <v>0.0258</v>
       </c>
       <c r="J4" s="50" t="n">
         <v>-0.07210569999999999</v>
@@ -25344,18 +25356,18 @@
         </is>
       </c>
       <c r="F5" s="47" t="n">
-        <v>34.05</v>
+        <v>34.86</v>
       </c>
       <c r="G5" s="45" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H5" s="47" t="n">
-        <v>0.26</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H5" s="56" t="n">
+        <v>0.8100000000000001</v>
       </c>
       <c r="I5" s="49" t="n">
-        <v>0.0077</v>
+        <v>0.0238</v>
       </c>
       <c r="J5" s="48" t="n">
         <v>-0.07485287</v>
@@ -25418,18 +25430,18 @@
         </is>
       </c>
       <c r="F6" s="43" t="n">
-        <v>50</v>
+        <v>53.15</v>
       </c>
       <c r="G6" s="41" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H6" s="43" t="n">
-        <v>0.05</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H6" s="55" t="n">
+        <v>3.15</v>
       </c>
       <c r="I6" s="44" t="n">
-        <v>0.001</v>
+        <v>0.063</v>
       </c>
       <c r="J6" s="44" t="n">
         <v>0.04219119</v>
@@ -25488,18 +25500,18 @@
         </is>
       </c>
       <c r="F7" s="47" t="n">
-        <v>42.48</v>
+        <v>38.33</v>
       </c>
       <c r="G7" s="45" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H7" s="47" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="I7" s="49" t="n">
-        <v>0.004</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H7" s="54" t="n">
+        <v>-4.15</v>
+      </c>
+      <c r="I7" s="48" t="n">
+        <v>-0.0977</v>
       </c>
       <c r="J7" s="49" t="n">
         <v>0.05804878</v>
@@ -25562,18 +25574,18 @@
         </is>
       </c>
       <c r="F8" s="43" t="n">
-        <v>107.6</v>
+        <v>100.6</v>
       </c>
       <c r="G8" s="41" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H8" s="43" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I8" s="44" t="n">
-        <v>0.005600000000000001</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H8" s="52" t="n">
+        <v>-7</v>
+      </c>
+      <c r="I8" s="50" t="n">
+        <v>-0.06509999999999999</v>
       </c>
       <c r="J8" s="44" t="n">
         <v>0.00911528</v>
@@ -25632,18 +25644,18 @@
         </is>
       </c>
       <c r="F9" s="47" t="n">
-        <v>27.97</v>
+        <v>28.02</v>
       </c>
       <c r="G9" s="45" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H9" s="47" t="n">
-        <v>0.4</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H9" s="56" t="n">
+        <v>0.05</v>
       </c>
       <c r="I9" s="49" t="n">
-        <v>0.0145</v>
+        <v>0.0018</v>
       </c>
       <c r="J9" s="49" t="n">
         <v>0.05632139</v>
@@ -25706,18 +25718,18 @@
         </is>
       </c>
       <c r="F10" s="43" t="n">
-        <v>25.82</v>
+        <v>28.56</v>
       </c>
       <c r="G10" s="41" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H10" s="43" t="n">
-        <v>0.33</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H10" s="55" t="n">
+        <v>2.74</v>
       </c>
       <c r="I10" s="44" t="n">
-        <v>0.0129</v>
+        <v>0.1061</v>
       </c>
       <c r="J10" s="50" t="n">
         <v>-0.09624573</v>
@@ -25776,18 +25788,18 @@
         </is>
       </c>
       <c r="F11" s="47" t="n">
-        <v>50</v>
+        <v>53.15</v>
       </c>
       <c r="G11" s="45" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H11" s="47" t="n">
-        <v>0.05</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H11" s="56" t="n">
+        <v>3.15</v>
       </c>
       <c r="I11" s="49" t="n">
-        <v>0.001</v>
+        <v>0.063</v>
       </c>
       <c r="J11" s="49" t="n">
         <v>0.04219119</v>
@@ -25846,18 +25858,18 @@
         </is>
       </c>
       <c r="F12" s="43" t="n">
-        <v>98.45</v>
+        <v>108.3</v>
       </c>
       <c r="G12" s="41" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H12" s="43" t="n">
-        <v>1.8</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H12" s="55" t="n">
+        <v>9.85</v>
       </c>
       <c r="I12" s="44" t="n">
-        <v>0.0186</v>
+        <v>0.1001</v>
       </c>
       <c r="J12" s="50" t="n">
         <v>-0.04014465</v>
@@ -25916,18 +25928,18 @@
         </is>
       </c>
       <c r="F13" s="47" t="n">
-        <v>83.95</v>
+        <v>87.5</v>
       </c>
       <c r="G13" s="45" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H13" s="47" t="n">
-        <v>0.6</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H13" s="56" t="n">
+        <v>3.55</v>
       </c>
       <c r="I13" s="49" t="n">
-        <v>0.0072</v>
+        <v>0.0423</v>
       </c>
       <c r="J13" s="48" t="n">
         <v>-0.11655405</v>
@@ -25986,18 +25998,18 @@
         </is>
       </c>
       <c r="F14" s="43" t="n">
-        <v>64.95</v>
+        <v>66.2</v>
       </c>
       <c r="G14" s="41" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H14" s="43" t="n">
-        <v>0.6</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H14" s="55" t="n">
+        <v>1.25</v>
       </c>
       <c r="I14" s="44" t="n">
-        <v>0.009300000000000001</v>
+        <v>0.0192</v>
       </c>
       <c r="J14" s="44" t="n">
         <v>0.03063547</v>
@@ -26056,18 +26068,18 @@
         </is>
       </c>
       <c r="F15" s="47" t="n">
-        <v>44.35</v>
+        <v>46.6</v>
       </c>
       <c r="G15" s="45" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H15" s="47" t="n">
-        <v>0.17</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H15" s="56" t="n">
+        <v>2.25</v>
       </c>
       <c r="I15" s="49" t="n">
-        <v>0.0038</v>
+        <v>0.0507</v>
       </c>
       <c r="J15" s="48" t="n">
         <v>-0.04295893000000001</v>
@@ -26126,25 +26138,25 @@
         </is>
       </c>
       <c r="F16" s="43" t="n">
-        <v>15.01</v>
+        <v>14.4</v>
       </c>
       <c r="G16" s="41" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H16" s="43" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="I16" s="44" t="n">
-        <v>0.004699999999999999</v>
-      </c>
-      <c r="J16" s="52" t="inlineStr"/>
-      <c r="K16" s="52" t="inlineStr"/>
-      <c r="L16" s="52" t="inlineStr"/>
-      <c r="M16" s="52" t="inlineStr"/>
-      <c r="N16" s="52" t="inlineStr"/>
-      <c r="O16" s="52" t="inlineStr"/>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H16" s="52" t="n">
+        <v>-0.61</v>
+      </c>
+      <c r="I16" s="50" t="n">
+        <v>-0.0406</v>
+      </c>
+      <c r="J16" s="53" t="inlineStr"/>
+      <c r="K16" s="53" t="inlineStr"/>
+      <c r="L16" s="53" t="inlineStr"/>
+      <c r="M16" s="53" t="inlineStr"/>
+      <c r="N16" s="53" t="inlineStr"/>
+      <c r="O16" s="53" t="inlineStr"/>
       <c r="P16" s="41" t="inlineStr">
         <is>
           <t>月配</t>
@@ -26316,18 +26328,18 @@
         </is>
       </c>
       <c r="F2" s="43" t="n">
-        <v>56.66</v>
+        <v>56.22</v>
       </c>
       <c r="G2" s="43" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H2" s="43" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="I2" s="44" t="n">
-        <v>0.0059</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H2" s="52" t="n">
+        <v>-0.44</v>
+      </c>
+      <c r="I2" s="50" t="n">
+        <v>-0.007800000000000001</v>
       </c>
       <c r="J2" s="44" t="n">
         <v>0.06641135000000001</v>
@@ -26390,18 +26402,18 @@
         </is>
       </c>
       <c r="F3" s="47" t="n">
-        <v>9.875299999999999</v>
+        <v>9.790900000000001</v>
       </c>
       <c r="G3" s="47" t="inlineStr">
         <is>
-          <t>10/15</t>
-        </is>
-      </c>
-      <c r="H3" s="47" t="n">
-        <v>0.09329999999999999</v>
-      </c>
-      <c r="I3" s="49" t="n">
-        <v>0.0095</v>
+          <t>10/16</t>
+        </is>
+      </c>
+      <c r="H3" s="54" t="n">
+        <v>-0.0844</v>
+      </c>
+      <c r="I3" s="48" t="n">
+        <v>-0.008500000000000001</v>
       </c>
       <c r="J3" s="48" t="n">
         <v>-0.02359118</v>
@@ -26464,18 +26476,18 @@
         </is>
       </c>
       <c r="F4" s="43" t="n">
-        <v>7.8916</v>
+        <v>7.8925</v>
       </c>
       <c r="G4" s="43" t="inlineStr">
         <is>
-          <t>10/15</t>
-        </is>
-      </c>
-      <c r="H4" s="43" t="n">
-        <v>0.0584</v>
+          <t>10/16</t>
+        </is>
+      </c>
+      <c r="H4" s="55" t="n">
+        <v>0.0009</v>
       </c>
       <c r="I4" s="44" t="n">
-        <v>0.0075</v>
+        <v>0.0001</v>
       </c>
       <c r="J4" s="50" t="n">
         <v>-0.01326918</v>
@@ -26538,18 +26550,18 @@
         </is>
       </c>
       <c r="F5" s="47" t="n">
-        <v>8.450900000000001</v>
+        <v>8.444000000000001</v>
       </c>
       <c r="G5" s="47" t="inlineStr">
         <is>
-          <t>10/15</t>
-        </is>
-      </c>
-      <c r="H5" s="47" t="n">
-        <v>0.115</v>
-      </c>
-      <c r="I5" s="49" t="n">
-        <v>0.0138</v>
+          <t>10/16</t>
+        </is>
+      </c>
+      <c r="H5" s="54" t="n">
+        <v>-0.0069</v>
+      </c>
+      <c r="I5" s="48" t="n">
+        <v>-0.0008</v>
       </c>
       <c r="J5" s="48" t="n">
         <v>-0.04286634</v>
@@ -26612,18 +26624,18 @@
         </is>
       </c>
       <c r="F6" s="43" t="n">
-        <v>9.8651</v>
+        <v>9.780799999999999</v>
       </c>
       <c r="G6" s="43" t="inlineStr">
         <is>
-          <t>10/15</t>
-        </is>
-      </c>
-      <c r="H6" s="43" t="n">
-        <v>0.09320000000000001</v>
-      </c>
-      <c r="I6" s="44" t="n">
-        <v>0.0095</v>
+          <t>10/16</t>
+        </is>
+      </c>
+      <c r="H6" s="52" t="n">
+        <v>-0.0843</v>
+      </c>
+      <c r="I6" s="50" t="n">
+        <v>-0.008500000000000001</v>
       </c>
       <c r="J6" s="50" t="n">
         <v>-0.02358716</v>
@@ -26686,18 +26698,18 @@
         </is>
       </c>
       <c r="F7" s="47" t="n">
-        <v>8.448600000000001</v>
+        <v>8.441599999999999</v>
       </c>
       <c r="G7" s="47" t="inlineStr">
         <is>
-          <t>10/15</t>
-        </is>
-      </c>
-      <c r="H7" s="47" t="n">
-        <v>0.115</v>
-      </c>
-      <c r="I7" s="49" t="n">
-        <v>0.0138</v>
+          <t>10/16</t>
+        </is>
+      </c>
+      <c r="H7" s="54" t="n">
+        <v>-0.007</v>
+      </c>
+      <c r="I7" s="48" t="n">
+        <v>-0.0008</v>
       </c>
       <c r="J7" s="48" t="n">
         <v>-0.04286672</v>
@@ -26760,18 +26772,18 @@
         </is>
       </c>
       <c r="F8" s="43" t="n">
-        <v>7.9185</v>
+        <v>7.9194</v>
       </c>
       <c r="G8" s="43" t="inlineStr">
         <is>
-          <t>10/15</t>
-        </is>
-      </c>
-      <c r="H8" s="43" t="n">
-        <v>0.0586</v>
+          <t>10/16</t>
+        </is>
+      </c>
+      <c r="H8" s="55" t="n">
+        <v>0.0009</v>
       </c>
       <c r="I8" s="44" t="n">
-        <v>0.0075</v>
+        <v>0.0001</v>
       </c>
       <c r="J8" s="50" t="n">
         <v>-0.01325601</v>
@@ -26834,18 +26846,18 @@
         </is>
       </c>
       <c r="F9" s="47" t="n">
-        <v>85.62</v>
+        <v>84.95999999999999</v>
       </c>
       <c r="G9" s="47" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H9" s="47" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I9" s="49" t="n">
-        <v>0.0059</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H9" s="54" t="n">
+        <v>-0.66</v>
+      </c>
+      <c r="I9" s="48" t="n">
+        <v>-0.0077</v>
       </c>
       <c r="J9" s="49" t="n">
         <v>0.06664248</v>
@@ -26908,18 +26920,18 @@
         </is>
       </c>
       <c r="F10" s="43" t="n">
-        <v>175.58</v>
+        <v>174.47</v>
       </c>
       <c r="G10" s="43" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H10" s="43" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="I10" s="44" t="n">
-        <v>0.0033</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H10" s="52" t="n">
+        <v>-1.11</v>
+      </c>
+      <c r="I10" s="50" t="n">
+        <v>-0.0063</v>
       </c>
       <c r="J10" s="50" t="n">
         <v>-0.04380673</v>
@@ -26982,18 +26994,18 @@
         </is>
       </c>
       <c r="F11" s="47" t="n">
-        <v>116.02</v>
+        <v>115.17</v>
       </c>
       <c r="G11" s="47" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H11" s="47" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="I11" s="49" t="n">
-        <v>0.0024</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H11" s="54" t="n">
+        <v>-0.85</v>
+      </c>
+      <c r="I11" s="48" t="n">
+        <v>-0.0073</v>
       </c>
       <c r="J11" s="49" t="n">
         <v>0.00866128</v>
@@ -27052,18 +27064,18 @@
         </is>
       </c>
       <c r="F12" s="43" t="n">
-        <v>352.98</v>
+        <v>350.57</v>
       </c>
       <c r="G12" s="43" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H12" s="43" t="n">
-        <v>-0.57</v>
+          <t>10/19</t>
+        </is>
+      </c>
+      <c r="H12" s="52" t="n">
+        <v>-2.41</v>
       </c>
       <c r="I12" s="50" t="n">
-        <v>-0.0016</v>
+        <v>-0.0068</v>
       </c>
       <c r="J12" s="44" t="n">
         <v>0.04333726</v>

</xml_diff>

<commit_message>
chore: 自動更新最新基金與ETF數據 (2026-10-20 15:44:27)
</commit_message>
<xml_diff>
--- a/國泰投信_人氣ETF與熱門基金分析.xlsx
+++ b/國泰投信_人氣ETF與熱門基金分析.xlsx
@@ -368,13 +368,13 @@
     <xf numFmtId="10" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="4" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="4" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2814,7 +2814,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="H7" s="23" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.7</v>
       </c>
       <c r="I7" s="25" t="n">
         <v>0</v>
@@ -2862,7 +2862,7 @@
         <v>42.8</v>
       </c>
       <c r="H8" s="29" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.5</v>
       </c>
       <c r="I8" s="31" t="n">
         <v>0</v>
@@ -4502,7 +4502,7 @@
         <v>0.0567</v>
       </c>
       <c r="H40" s="32" t="n">
-        <v/>
+        <v>15.48</v>
       </c>
       <c r="I40" s="27" t="inlineStr">
         <is>
@@ -4514,9 +4514,9 @@
           <t>2026/11/12</t>
         </is>
       </c>
-      <c r="K40" s="26" t="inlineStr">
-        <is>
-          <t>資料不足</t>
+      <c r="K40" s="33" t="inlineStr">
+        <is>
+          <t>尚未填息 (貼息中)</t>
         </is>
       </c>
       <c r="L40" s="34" t="n">
@@ -5132,7 +5132,7 @@
         <v>0.0579</v>
       </c>
       <c r="H50" s="32" t="n">
-        <v/>
+        <v>34.05</v>
       </c>
       <c r="I50" s="27" t="inlineStr">
         <is>
@@ -5144,9 +5144,9 @@
           <t>2026/11/12</t>
         </is>
       </c>
-      <c r="K50" s="26" t="inlineStr">
-        <is>
-          <t>資料不足</t>
+      <c r="K50" s="33" t="inlineStr">
+        <is>
+          <t>尚未填息 (貼息中)</t>
         </is>
       </c>
       <c r="L50" s="34" t="n">
@@ -13145,16 +13145,16 @@
         <v>0</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>0.5085999999999999</v>
+        <v>0.5079</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.5085999999999999</v>
+        <v>0.5079</v>
       </c>
       <c r="G6" s="29" t="n">
-        <v>0.3591</v>
+        <v>0.3598000000000001</v>
       </c>
       <c r="H6" s="29" t="n">
-        <v>0.1036</v>
+        <v>0.1039</v>
       </c>
       <c r="I6" s="27" t="n">
         <v>0</v>
@@ -13166,7 +13166,7 @@
       </c>
       <c r="K6" s="27" t="inlineStr">
         <is>
-          <t>中信金(10.16%), 廣達(8.63%), 國泰金(6.57%)</t>
+          <t>中信金(10.22%), 廣達(8.51%), 國泰金(6.54%)</t>
         </is>
       </c>
     </row>
@@ -13322,19 +13322,19 @@
         </is>
       </c>
       <c r="D10" s="29" t="n">
-        <v>0.3724</v>
+        <v>0.3937</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.4019</v>
+        <v>0.4217000000000001</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>0.7743000000000001</v>
+        <v>0.8154</v>
       </c>
       <c r="G10" s="29" t="n">
-        <v>0.1302</v>
+        <v>0.1362</v>
       </c>
       <c r="H10" s="29" t="n">
-        <v>0.033</v>
+        <v>0.0348</v>
       </c>
       <c r="I10" s="27" t="n">
         <v>0</v>
@@ -13346,7 +13346,7 @@
       </c>
       <c r="K10" s="27" t="inlineStr">
         <is>
-          <t>台積電(37.24%), 聯發科(6.35%), 台達電(3.59%)</t>
+          <t>台積電(39.37%), 聯發科(6.64%), 台達電(3.8%)</t>
         </is>
       </c>
     </row>
@@ -13427,7 +13427,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="27" t="n">
-        <v>0.9996999999999998</v>
+        <v>0.9995000000000001</v>
       </c>
       <c r="J12" s="27" t="inlineStr">
         <is>
@@ -13436,7 +13436,7 @@
       </c>
       <c r="K12" s="27" t="inlineStr">
         <is>
-          <t>Apple Inc.(17.5%), Microsoft Corp(14.17%), AMAZON.COM INC(8.92%)</t>
+          <t>Apple Inc.(17.36%), Microsoft Corp(14.2%), AMAZON.COM INC(9.31%)</t>
         </is>
       </c>
     </row>
@@ -13562,7 +13562,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="21" t="n">
-        <v>0.9980999999999999</v>
+        <v>0.9987</v>
       </c>
       <c r="J15" s="21" t="inlineStr">
         <is>
@@ -13571,7 +13571,7 @@
       </c>
       <c r="K15" s="21" t="inlineStr">
         <is>
-          <t>NVIDIA CORPORATION(12.07%), BROADCOM INC(9.2%), Micron Technology Inc(7.6%)</t>
+          <t>NVIDIA CORPORATION(12.04%), BROADCOM INC(9.22%), Micron Technology Inc(7.71%)</t>
         </is>
       </c>
     </row>
@@ -13607,7 +13607,7 @@
         <v>0</v>
       </c>
       <c r="I16" s="27" t="n">
-        <v>0.9868000000000027</v>
+        <v>0.9869000000000027</v>
       </c>
       <c r="J16" s="27" t="inlineStr">
         <is>
@@ -13616,7 +13616,7 @@
       </c>
       <c r="K16" s="27" t="inlineStr">
         <is>
-          <t>Apple Inc.(9.33%), Microsoft Corp(9.22%), NVIDIA CORPORATION(8.2%)</t>
+          <t>Apple Inc.(9.2%), Microsoft Corp(9.18%), NVIDIA CORPORATION(8.21%)</t>
         </is>
       </c>
     </row>
@@ -13640,10 +13640,10 @@
         <v>0</v>
       </c>
       <c r="E17" s="23" t="n">
-        <v>0.0346</v>
+        <v>0.0341</v>
       </c>
       <c r="F17" s="23" t="n">
-        <v>0.0346</v>
+        <v>0.0341</v>
       </c>
       <c r="G17" s="25" t="n">
         <v>0</v>
@@ -13652,7 +13652,7 @@
         <v>0</v>
       </c>
       <c r="I17" s="21" t="n">
-        <v>0.9529999999999998</v>
+        <v>0.9521999999999999</v>
       </c>
       <c r="J17" s="21" t="inlineStr">
         <is>
@@ -13661,7 +13661,7 @@
       </c>
       <c r="K17" s="21" t="inlineStr">
         <is>
-          <t>ADV MICRO DEVICES(25.83%), NVIDIA CORPORATION(14.41%), TESLA, INC.(12.01%)</t>
+          <t>ADV MICRO DEVICES(25.97%), NVIDIA CORPORATION(14.43%), TESLA, INC.(12.32%)</t>
         </is>
       </c>
     </row>
@@ -14679,11 +14679,11 @@
         </is>
       </c>
       <c r="H43" s="23" t="n">
-        <v>0.1016</v>
+        <v>0.1022</v>
       </c>
       <c r="I43" s="21" t="inlineStr">
         <is>
-          <t>926,187,000</t>
+          <t>928,342,000</t>
         </is>
       </c>
     </row>
@@ -14722,11 +14722,11 @@
         </is>
       </c>
       <c r="H44" s="29" t="n">
-        <v>0.0863</v>
+        <v>0.0851</v>
       </c>
       <c r="I44" s="27" t="inlineStr">
         <is>
-          <t>179,841,000</t>
+          <t>180,259,000</t>
         </is>
       </c>
     </row>
@@ -14765,11 +14765,11 @@
         </is>
       </c>
       <c r="H45" s="23" t="n">
-        <v>0.06570000000000001</v>
+        <v>0.0654</v>
       </c>
       <c r="I45" s="21" t="inlineStr">
         <is>
-          <t>379,840,486</t>
+          <t>380,724,486</t>
         </is>
       </c>
     </row>
@@ -14808,11 +14808,11 @@
         </is>
       </c>
       <c r="H46" s="29" t="n">
-        <v>0.0585</v>
+        <v>0.0576</v>
       </c>
       <c r="I46" s="27" t="inlineStr">
         <is>
-          <t>39,520,000</t>
+          <t>39,612,000</t>
         </is>
       </c>
     </row>
@@ -14851,11 +14851,11 @@
         </is>
       </c>
       <c r="H47" s="25" t="n">
-        <v>0.0446</v>
+        <v>0.0445</v>
       </c>
       <c r="I47" s="21" t="inlineStr">
         <is>
-          <t>112,722,000</t>
+          <t>113,112,000</t>
         </is>
       </c>
     </row>
@@ -14894,11 +14894,11 @@
         </is>
       </c>
       <c r="H48" s="31" t="n">
-        <v>0.0382</v>
+        <v>0.0385</v>
       </c>
       <c r="I48" s="27" t="inlineStr">
         <is>
-          <t>604,527,270</t>
+          <t>605,933,270</t>
         </is>
       </c>
     </row>
@@ -14937,11 +14937,11 @@
         </is>
       </c>
       <c r="H49" s="25" t="n">
-        <v>0.0377</v>
+        <v>0.03759999999999999</v>
       </c>
       <c r="I49" s="21" t="inlineStr">
         <is>
-          <t>190,401,000</t>
+          <t>190,844,000</t>
         </is>
       </c>
     </row>
@@ -14980,11 +14980,11 @@
         </is>
       </c>
       <c r="H50" s="31" t="n">
-        <v>0.0327</v>
+        <v>0.0329</v>
       </c>
       <c r="I50" s="27" t="inlineStr">
         <is>
-          <t>449,396,250</t>
+          <t>450,442,250</t>
         </is>
       </c>
     </row>
@@ -15027,7 +15027,7 @@
       </c>
       <c r="I51" s="21" t="inlineStr">
         <is>
-          <t>5,167,000</t>
+          <t>5,179,000</t>
         </is>
       </c>
     </row>
@@ -15066,11 +15066,11 @@
         </is>
       </c>
       <c r="H52" s="31" t="n">
-        <v>0.0323</v>
+        <v>0.0325</v>
       </c>
       <c r="I52" s="27" t="inlineStr">
         <is>
-          <t>27,829,000</t>
+          <t>27,834,000</t>
         </is>
       </c>
     </row>
@@ -16239,11 +16239,11 @@
         </is>
       </c>
       <c r="H83" s="23" t="n">
-        <v>0.3724</v>
+        <v>0.3937</v>
       </c>
       <c r="I83" s="21" t="inlineStr">
         <is>
-          <t>14,797,702</t>
+          <t>14,811,446</t>
         </is>
       </c>
     </row>
@@ -16282,11 +16282,11 @@
         </is>
       </c>
       <c r="H84" s="29" t="n">
-        <v>0.0635</v>
+        <v>0.0664</v>
       </c>
       <c r="I84" s="27" t="inlineStr">
         <is>
-          <t>1,437,355</t>
+          <t>1,438,711</t>
         </is>
       </c>
     </row>
@@ -16325,11 +16325,11 @@
         </is>
       </c>
       <c r="H85" s="25" t="n">
-        <v>0.0359</v>
+        <v>0.038</v>
       </c>
       <c r="I85" s="21" t="inlineStr">
         <is>
-          <t>2,108,747</t>
+          <t>2,110,739</t>
         </is>
       </c>
     </row>
@@ -16368,11 +16368,11 @@
         </is>
       </c>
       <c r="H86" s="31" t="n">
-        <v>0.0313</v>
+        <v>0.0325</v>
       </c>
       <c r="I86" s="27" t="inlineStr">
         <is>
-          <t>12,348,687</t>
+          <t>12,360,359</t>
         </is>
       </c>
     </row>
@@ -16411,11 +16411,11 @@
         </is>
       </c>
       <c r="H87" s="25" t="n">
-        <v>0.0283</v>
+        <v>0.0299</v>
       </c>
       <c r="I87" s="21" t="inlineStr">
         <is>
-          <t>4,056,092</t>
+          <t>4,059,924</t>
         </is>
       </c>
     </row>
@@ -16454,11 +16454,11 @@
         </is>
       </c>
       <c r="H88" s="31" t="n">
-        <v>0.0203</v>
+        <v>0.0213</v>
       </c>
       <c r="I88" s="27" t="inlineStr">
         <is>
-          <t>378,003</t>
+          <t>378,359</t>
         </is>
       </c>
     </row>
@@ -16497,11 +16497,11 @@
         </is>
       </c>
       <c r="H89" s="25" t="n">
-        <v>0.0199</v>
+        <v>0.0208</v>
       </c>
       <c r="I89" s="21" t="inlineStr">
         <is>
-          <t>14,390,909</t>
+          <t>14,404,513</t>
         </is>
       </c>
     </row>
@@ -16540,11 +16540,11 @@
         </is>
       </c>
       <c r="H90" s="31" t="n">
-        <v>0.0178</v>
+        <v>0.0184</v>
       </c>
       <c r="I90" s="27" t="inlineStr">
         <is>
-          <t>10,585,154</t>
+          <t>10,595,170</t>
         </is>
       </c>
     </row>
@@ -16583,11 +16583,11 @@
         </is>
       </c>
       <c r="H91" s="25" t="n">
-        <v>0.0168</v>
+        <v>0.0176</v>
       </c>
       <c r="I91" s="21" t="inlineStr">
         <is>
-          <t>5,260,206</t>
+          <t>5,265,178</t>
         </is>
       </c>
     </row>
@@ -16612,25 +16612,25 @@
       </c>
       <c r="E92" s="26" t="inlineStr">
         <is>
-          <t>2891</t>
+          <t>3017</t>
         </is>
       </c>
       <c r="F92" s="27" t="inlineStr">
         <is>
-          <t>中信金</t>
+          <t>奇鋐</t>
         </is>
       </c>
       <c r="G92" s="27" t="inlineStr">
         <is>
-          <t>金融保險</t>
+          <t>科技電子</t>
         </is>
       </c>
       <c r="H92" s="31" t="n">
-        <v>0.0161</v>
+        <v>0.017</v>
       </c>
       <c r="I92" s="27" t="inlineStr">
         <is>
-          <t>20,998,007</t>
+          <t>465,334</t>
         </is>
       </c>
     </row>
@@ -16669,11 +16669,11 @@
         </is>
       </c>
       <c r="H93" s="23" t="n">
-        <v>0.175</v>
+        <v>0.1736</v>
       </c>
       <c r="I93" s="21" t="inlineStr">
         <is>
-          <t>40,189</t>
+          <t>39,519</t>
         </is>
       </c>
     </row>
@@ -16712,11 +16712,11 @@
         </is>
       </c>
       <c r="H94" s="29" t="n">
-        <v>0.1417</v>
+        <v>0.142</v>
       </c>
       <c r="I94" s="27" t="inlineStr">
         <is>
-          <t>21,135</t>
+          <t>20,785</t>
         </is>
       </c>
     </row>
@@ -16755,11 +16755,11 @@
         </is>
       </c>
       <c r="H95" s="23" t="n">
-        <v>0.0892</v>
+        <v>0.0931</v>
       </c>
       <c r="I95" s="21" t="inlineStr">
         <is>
-          <t>28,146</t>
+          <t>27,688</t>
         </is>
       </c>
     </row>
@@ -16798,11 +16798,11 @@
         </is>
       </c>
       <c r="H96" s="29" t="n">
-        <v>0.0725</v>
+        <v>0.0728</v>
       </c>
       <c r="I96" s="27" t="inlineStr">
         <is>
-          <t>16,787</t>
+          <t>16,513</t>
         </is>
       </c>
     </row>
@@ -16841,11 +16841,11 @@
         </is>
       </c>
       <c r="H97" s="23" t="n">
-        <v>0.0568</v>
+        <v>0.0562</v>
       </c>
       <c r="I97" s="21" t="inlineStr">
         <is>
-          <t>6,320</t>
+          <t>6,217</t>
         </is>
       </c>
     </row>
@@ -16884,11 +16884,11 @@
         </is>
       </c>
       <c r="H98" s="31" t="n">
-        <v>0.0366</v>
+        <v>0.0378</v>
       </c>
       <c r="I98" s="27" t="inlineStr">
         <is>
-          <t>8,146</t>
+          <t>8,014</t>
         </is>
       </c>
     </row>
@@ -16927,11 +16927,11 @@
         </is>
       </c>
       <c r="H99" s="25" t="n">
-        <v>0.0335</v>
+        <v>0.0326</v>
       </c>
       <c r="I99" s="21" t="inlineStr">
         <is>
-          <t>7,768</t>
+          <t>7,641</t>
         </is>
       </c>
     </row>
@@ -16970,7 +16970,7 @@
         </is>
       </c>
       <c r="H100" s="31" t="n">
-        <v>0.0295</v>
+        <v>0.0302</v>
       </c>
       <c r="I100" s="27" t="inlineStr">
         <is>
@@ -17013,11 +17013,11 @@
         </is>
       </c>
       <c r="H101" s="25" t="n">
-        <v>0.0248</v>
+        <v>0.0246</v>
       </c>
       <c r="I101" s="21" t="inlineStr">
         <is>
-          <t>4,853</t>
+          <t>4,774</t>
         </is>
       </c>
     </row>
@@ -17056,11 +17056,11 @@
         </is>
       </c>
       <c r="H102" s="31" t="n">
-        <v>0.0191</v>
+        <v>0.0189</v>
       </c>
       <c r="I102" s="27" t="inlineStr">
         <is>
-          <t>12,657</t>
+          <t>12,451</t>
         </is>
       </c>
     </row>
@@ -17959,11 +17959,11 @@
         </is>
       </c>
       <c r="H123" s="23" t="n">
-        <v>0.1207</v>
+        <v>0.1204</v>
       </c>
       <c r="I123" s="21" t="inlineStr">
         <is>
-          <t>1,270,494</t>
+          <t>1,276,794</t>
         </is>
       </c>
     </row>
@@ -18002,11 +18002,11 @@
         </is>
       </c>
       <c r="H124" s="29" t="n">
-        <v>0.092</v>
+        <v>0.0922</v>
       </c>
       <c r="I124" s="27" t="inlineStr">
         <is>
-          <t>631,201</t>
+          <t>634,331</t>
         </is>
       </c>
     </row>
@@ -18045,11 +18045,11 @@
         </is>
       </c>
       <c r="H125" s="23" t="n">
-        <v>0.076</v>
+        <v>0.0771</v>
       </c>
       <c r="I125" s="21" t="inlineStr">
         <is>
-          <t>195,057</t>
+          <t>196,024</t>
         </is>
       </c>
     </row>
@@ -18088,11 +18088,11 @@
         </is>
       </c>
       <c r="H126" s="31" t="n">
-        <v>0.0466</v>
+        <v>0.0467</v>
       </c>
       <c r="I126" s="27" t="inlineStr">
         <is>
-          <t>198,639</t>
+          <t>199,624</t>
         </is>
       </c>
     </row>
@@ -18117,12 +18117,12 @@
       </c>
       <c r="E127" s="20" t="inlineStr">
         <is>
-          <t>ADI.US</t>
+          <t>MRVL.US</t>
         </is>
       </c>
       <c r="F127" s="21" t="inlineStr">
         <is>
-          <t>ANALOG DEVICES INC</t>
+          <t>MARVELL TECH GROUP</t>
         </is>
       </c>
       <c r="G127" s="21" t="inlineStr">
@@ -18131,11 +18131,11 @@
         </is>
       </c>
       <c r="H127" s="25" t="n">
-        <v>0.0453</v>
+        <v>0.0457</v>
       </c>
       <c r="I127" s="21" t="inlineStr">
         <is>
-          <t>258,197</t>
+          <t>443,954</t>
         </is>
       </c>
     </row>
@@ -18160,12 +18160,12 @@
       </c>
       <c r="E128" s="26" t="inlineStr">
         <is>
-          <t>MRVL.US</t>
+          <t>ADI.US</t>
         </is>
       </c>
       <c r="F128" s="27" t="inlineStr">
         <is>
-          <t>MARVELL TECH GROUP</t>
+          <t>ANALOG DEVICES INC</t>
         </is>
       </c>
       <c r="G128" s="27" t="inlineStr">
@@ -18174,11 +18174,11 @@
         </is>
       </c>
       <c r="H128" s="31" t="n">
-        <v>0.0446</v>
+        <v>0.0445</v>
       </c>
       <c r="I128" s="27" t="inlineStr">
         <is>
-          <t>441,763</t>
+          <t>259,478</t>
         </is>
       </c>
     </row>
@@ -18217,11 +18217,11 @@
         </is>
       </c>
       <c r="H129" s="25" t="n">
-        <v>0.04389999999999999</v>
+        <v>0.0432</v>
       </c>
       <c r="I129" s="21" t="inlineStr">
         <is>
-          <t>358,375</t>
+          <t>360,152</t>
         </is>
       </c>
     </row>
@@ -18246,12 +18246,12 @@
       </c>
       <c r="E130" s="26" t="inlineStr">
         <is>
-          <t>QCOM.US</t>
+          <t>INTC.US</t>
         </is>
       </c>
       <c r="F130" s="27" t="inlineStr">
         <is>
-          <t>QUALCOMM INC</t>
+          <t>Intel Corp</t>
         </is>
       </c>
       <c r="G130" s="27" t="inlineStr">
@@ -18260,11 +18260,11 @@
         </is>
       </c>
       <c r="H130" s="31" t="n">
-        <v>0.04190000000000001</v>
+        <v>0.042</v>
       </c>
       <c r="I130" s="27" t="inlineStr">
         <is>
-          <t>548,472</t>
+          <t>1,049,796</t>
         </is>
       </c>
     </row>
@@ -18289,12 +18289,12 @@
       </c>
       <c r="E131" s="20" t="inlineStr">
         <is>
-          <t>INTC.US</t>
+          <t>QCOM.US</t>
         </is>
       </c>
       <c r="F131" s="21" t="inlineStr">
         <is>
-          <t>Intel Corp</t>
+          <t>QUALCOMM INC</t>
         </is>
       </c>
       <c r="G131" s="21" t="inlineStr">
@@ -18307,7 +18307,7 @@
       </c>
       <c r="I131" s="21" t="inlineStr">
         <is>
-          <t>1,044,616</t>
+          <t>551,192</t>
         </is>
       </c>
     </row>
@@ -18346,11 +18346,11 @@
         </is>
       </c>
       <c r="H132" s="31" t="n">
-        <v>0.0412</v>
+        <v>0.0413</v>
       </c>
       <c r="I132" s="27" t="inlineStr">
         <is>
-          <t>225,136</t>
+          <t>226,253</t>
         </is>
       </c>
     </row>
@@ -18389,11 +18389,11 @@
         </is>
       </c>
       <c r="H133" s="23" t="n">
-        <v>0.09329999999999999</v>
+        <v>0.092</v>
       </c>
       <c r="I133" s="21" t="inlineStr">
         <is>
-          <t>50,314</t>
+          <t>50,599</t>
         </is>
       </c>
     </row>
@@ -18432,11 +18432,11 @@
         </is>
       </c>
       <c r="H134" s="29" t="n">
-        <v>0.0922</v>
+        <v>0.09179999999999999</v>
       </c>
       <c r="I134" s="27" t="inlineStr">
         <is>
-          <t>32,271</t>
+          <t>32,454</t>
         </is>
       </c>
     </row>
@@ -18475,11 +18475,11 @@
         </is>
       </c>
       <c r="H135" s="23" t="n">
-        <v>0.08199999999999999</v>
+        <v>0.08210000000000001</v>
       </c>
       <c r="I135" s="21" t="inlineStr">
         <is>
-          <t>70,935</t>
+          <t>71,336</t>
         </is>
       </c>
     </row>
@@ -18518,11 +18518,11 @@
         </is>
       </c>
       <c r="H136" s="29" t="n">
-        <v>0.0698</v>
+        <v>0.0702</v>
       </c>
       <c r="I136" s="27" t="inlineStr">
         <is>
-          <t>39,344</t>
+          <t>39,567</t>
         </is>
       </c>
     </row>
@@ -18547,12 +18547,12 @@
       </c>
       <c r="E137" s="20" t="inlineStr">
         <is>
-          <t>META.US</t>
+          <t>GOOGL.US</t>
         </is>
       </c>
       <c r="F137" s="21" t="inlineStr">
         <is>
-          <t>Meta平台公司</t>
+          <t>ALPHABET CL A CMN</t>
         </is>
       </c>
       <c r="G137" s="21" t="inlineStr">
@@ -18561,11 +18561,11 @@
         </is>
       </c>
       <c r="H137" s="25" t="n">
-        <v>0.0492</v>
+        <v>0.0488</v>
       </c>
       <c r="I137" s="21" t="inlineStr">
         <is>
-          <t>12,850</t>
+          <t>26,743</t>
         </is>
       </c>
     </row>
@@ -18590,12 +18590,12 @@
       </c>
       <c r="E138" s="26" t="inlineStr">
         <is>
-          <t>GOOGL.US</t>
+          <t>META.US</t>
         </is>
       </c>
       <c r="F138" s="27" t="inlineStr">
         <is>
-          <t>ALPHABET CL A CMN</t>
+          <t>Meta平台公司</t>
         </is>
       </c>
       <c r="G138" s="27" t="inlineStr">
@@ -18604,11 +18604,11 @@
         </is>
       </c>
       <c r="H138" s="31" t="n">
-        <v>0.0489</v>
+        <v>0.0483</v>
       </c>
       <c r="I138" s="27" t="inlineStr">
         <is>
-          <t>26,592</t>
+          <t>12,922</t>
         </is>
       </c>
     </row>
@@ -18647,11 +18647,11 @@
         </is>
       </c>
       <c r="H139" s="25" t="n">
-        <v>0.0406</v>
+        <v>0.0408</v>
       </c>
       <c r="I139" s="21" t="inlineStr">
         <is>
-          <t>14,230</t>
+          <t>14,310</t>
         </is>
       </c>
     </row>
@@ -18676,12 +18676,12 @@
       </c>
       <c r="E140" s="26" t="inlineStr">
         <is>
-          <t>GOOG.US</t>
+          <t>MU.US</t>
         </is>
       </c>
       <c r="F140" s="27" t="inlineStr">
         <is>
-          <t>ALPHABET INC-CL C</t>
+          <t>Micron Technology Inc</t>
         </is>
       </c>
       <c r="G140" s="27" t="inlineStr">
@@ -18690,11 +18690,11 @@
         </is>
       </c>
       <c r="H140" s="31" t="n">
-        <v>0.0392</v>
+        <v>0.0394</v>
       </c>
       <c r="I140" s="27" t="inlineStr">
         <is>
-          <t>21,540</t>
+          <t>8,219</t>
         </is>
       </c>
     </row>
@@ -18719,12 +18719,12 @@
       </c>
       <c r="E141" s="20" t="inlineStr">
         <is>
-          <t>MU.US</t>
+          <t>GOOG.US</t>
         </is>
       </c>
       <c r="F141" s="21" t="inlineStr">
         <is>
-          <t>Micron Technology Inc</t>
+          <t>ALPHABET INC-CL C</t>
         </is>
       </c>
       <c r="G141" s="21" t="inlineStr">
@@ -18733,11 +18733,11 @@
         </is>
       </c>
       <c r="H141" s="25" t="n">
-        <v>0.0388</v>
+        <v>0.0391</v>
       </c>
       <c r="I141" s="21" t="inlineStr">
         <is>
-          <t>8,173</t>
+          <t>21,662</t>
         </is>
       </c>
     </row>
@@ -18776,11 +18776,11 @@
         </is>
       </c>
       <c r="H142" s="31" t="n">
-        <v>0.021</v>
+        <v>0.0213</v>
       </c>
       <c r="I142" s="27" t="inlineStr">
         <is>
-          <t>43,313</t>
+          <t>43,558</t>
         </is>
       </c>
     </row>
@@ -18819,7 +18819,7 @@
         </is>
       </c>
       <c r="H143" s="23" t="n">
-        <v>0.2583</v>
+        <v>0.2597</v>
       </c>
       <c r="I143" s="21" t="inlineStr">
         <is>
@@ -18862,7 +18862,7 @@
         </is>
       </c>
       <c r="H144" s="29" t="n">
-        <v>0.1441</v>
+        <v>0.1443</v>
       </c>
       <c r="I144" s="27" t="inlineStr">
         <is>
@@ -18905,7 +18905,7 @@
         </is>
       </c>
       <c r="H145" s="23" t="n">
-        <v>0.1201</v>
+        <v>0.1232</v>
       </c>
       <c r="I145" s="21" t="inlineStr">
         <is>
@@ -18948,7 +18948,7 @@
         </is>
       </c>
       <c r="H146" s="29" t="n">
-        <v>0.103</v>
+        <v>0.1016</v>
       </c>
       <c r="I146" s="27" t="inlineStr">
         <is>
@@ -18991,7 +18991,7 @@
         </is>
       </c>
       <c r="H147" s="23" t="n">
-        <v>0.0561</v>
+        <v>0.0549</v>
       </c>
       <c r="I147" s="21" t="inlineStr">
         <is>
@@ -19034,7 +19034,7 @@
         </is>
       </c>
       <c r="H148" s="31" t="n">
-        <v>0.042</v>
+        <v>0.04</v>
       </c>
       <c r="I148" s="27" t="inlineStr">
         <is>
@@ -19077,7 +19077,7 @@
         </is>
       </c>
       <c r="H149" s="25" t="n">
-        <v>0.0382</v>
+        <v>0.0375</v>
       </c>
       <c r="I149" s="21" t="inlineStr">
         <is>
@@ -19120,7 +19120,7 @@
         </is>
       </c>
       <c r="H150" s="31" t="n">
-        <v>0.0346</v>
+        <v>0.0341</v>
       </c>
       <c r="I150" s="27" t="inlineStr">
         <is>
@@ -19163,7 +19163,7 @@
         </is>
       </c>
       <c r="H151" s="25" t="n">
-        <v>0.0271</v>
+        <v>0.0269</v>
       </c>
       <c r="I151" s="21" t="inlineStr">
         <is>
@@ -19206,7 +19206,7 @@
         </is>
       </c>
       <c r="H152" s="31" t="n">
-        <v>0.0252</v>
+        <v>0.0251</v>
       </c>
       <c r="I152" s="27" t="inlineStr">
         <is>
@@ -23639,7 +23639,7 @@
         </is>
       </c>
       <c r="F2" s="43" t="n">
-        <v>100.6</v>
+        <v>103.45</v>
       </c>
       <c r="G2" s="44" t="n">
         <v>0.00911528</v>
@@ -23697,7 +23697,7 @@
         </is>
       </c>
       <c r="F3" s="47" t="n">
-        <v>108.3</v>
+        <v>96</v>
       </c>
       <c r="G3" s="48" t="n">
         <v>-0.04014465</v>
@@ -23987,7 +23987,7 @@
         </is>
       </c>
       <c r="F8" s="43" t="n">
-        <v>53.15</v>
+        <v>49.11</v>
       </c>
       <c r="G8" s="44" t="n">
         <v>0.04219119</v>
@@ -24045,7 +24045,7 @@
         </is>
       </c>
       <c r="F9" s="47" t="n">
-        <v>87.5</v>
+        <v>81</v>
       </c>
       <c r="G9" s="48" t="n">
         <v>-0.11655405</v>
@@ -24161,7 +24161,7 @@
         </is>
       </c>
       <c r="F11" s="47" t="n">
-        <v>38.33</v>
+        <v>39.56</v>
       </c>
       <c r="G11" s="49" t="n">
         <v>0.05804878</v>
@@ -24219,7 +24219,7 @@
         </is>
       </c>
       <c r="F12" s="43" t="n">
-        <v>30</v>
+        <v>34.88</v>
       </c>
       <c r="G12" s="44" t="n">
         <v>0.07029505</v>
@@ -24277,7 +24277,7 @@
         </is>
       </c>
       <c r="F13" s="47" t="n">
-        <v>46.6</v>
+        <v>43.4</v>
       </c>
       <c r="G13" s="48" t="n">
         <v>-0.04295893000000001</v>
@@ -24335,7 +24335,7 @@
         </is>
       </c>
       <c r="F14" s="43" t="n">
-        <v>66.2</v>
+        <v>63.7</v>
       </c>
       <c r="G14" s="44" t="n">
         <v>0.03063547</v>
@@ -24393,7 +24393,7 @@
         </is>
       </c>
       <c r="F15" s="47" t="n">
-        <v>28.02</v>
+        <v>27.98</v>
       </c>
       <c r="G15" s="49" t="n">
         <v>0.05632139</v>
@@ -24567,7 +24567,7 @@
         </is>
       </c>
       <c r="F18" s="43" t="n">
-        <v>28.56</v>
+        <v>25.76</v>
       </c>
       <c r="G18" s="50" t="n">
         <v>-0.09624573</v>
@@ -24857,7 +24857,7 @@
         </is>
       </c>
       <c r="F23" s="47" t="n">
-        <v>15.88</v>
+        <v>15.4</v>
       </c>
       <c r="G23" s="48" t="n">
         <v>-0.07210569999999999</v>
@@ -24915,7 +24915,7 @@
         </is>
       </c>
       <c r="F24" s="43" t="n">
-        <v>34.86</v>
+        <v>33.42</v>
       </c>
       <c r="G24" s="50" t="n">
         <v>-0.07485287</v>
@@ -24973,7 +24973,7 @@
         </is>
       </c>
       <c r="F25" s="47" t="n">
-        <v>14.4</v>
+        <v>14.61</v>
       </c>
       <c r="G25" s="51" t="inlineStr"/>
       <c r="H25" s="51" t="inlineStr"/>
@@ -25146,18 +25146,18 @@
         </is>
       </c>
       <c r="F2" s="43" t="n">
-        <v>14.4</v>
+        <v>14.61</v>
       </c>
       <c r="G2" s="41" t="inlineStr">
         <is>
-          <t>10/19</t>
+          <t>10/20</t>
         </is>
       </c>
       <c r="H2" s="52" t="n">
-        <v>-0.61</v>
+        <v>-0.24</v>
       </c>
       <c r="I2" s="50" t="n">
-        <v>-0.0406</v>
+        <v>-0.0162</v>
       </c>
       <c r="J2" s="53" t="inlineStr"/>
       <c r="K2" s="53" t="inlineStr"/>
@@ -25208,18 +25208,18 @@
         </is>
       </c>
       <c r="F3" s="47" t="n">
-        <v>30</v>
+        <v>34.88</v>
       </c>
       <c r="G3" s="45" t="inlineStr">
         <is>
-          <t>10/19</t>
+          <t>10/20</t>
         </is>
       </c>
       <c r="H3" s="54" t="n">
-        <v>-5.53</v>
-      </c>
-      <c r="I3" s="48" t="n">
-        <v>-0.1556</v>
+        <v>4.88</v>
+      </c>
+      <c r="I3" s="49" t="n">
+        <v>0.1627</v>
       </c>
       <c r="J3" s="49" t="n">
         <v>0.07029505</v>
@@ -25282,18 +25282,18 @@
         </is>
       </c>
       <c r="F4" s="43" t="n">
-        <v>15.88</v>
+        <v>15.4</v>
       </c>
       <c r="G4" s="41" t="inlineStr">
         <is>
-          <t>10/19</t>
-        </is>
-      </c>
-      <c r="H4" s="55" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="I4" s="44" t="n">
-        <v>0.0258</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H4" s="52" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="I4" s="50" t="n">
+        <v>-0.0019</v>
       </c>
       <c r="J4" s="50" t="n">
         <v>-0.07210569999999999</v>
@@ -25356,18 +25356,18 @@
         </is>
       </c>
       <c r="F5" s="47" t="n">
-        <v>34.86</v>
+        <v>33.42</v>
       </c>
       <c r="G5" s="45" t="inlineStr">
         <is>
-          <t>10/19</t>
-        </is>
-      </c>
-      <c r="H5" s="56" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="I5" s="49" t="n">
-        <v>0.0238</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H5" s="55" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="I5" s="48" t="n">
+        <v>-0.005699999999999999</v>
       </c>
       <c r="J5" s="48" t="n">
         <v>-0.07485287</v>
@@ -25430,18 +25430,18 @@
         </is>
       </c>
       <c r="F6" s="43" t="n">
-        <v>53.15</v>
+        <v>49.11</v>
       </c>
       <c r="G6" s="41" t="inlineStr">
         <is>
-          <t>10/19</t>
-        </is>
-      </c>
-      <c r="H6" s="55" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="I6" s="44" t="n">
-        <v>0.063</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H6" s="52" t="n">
+        <v>-4.04</v>
+      </c>
+      <c r="I6" s="50" t="n">
+        <v>-0.076</v>
       </c>
       <c r="J6" s="44" t="n">
         <v>0.04219119</v>
@@ -25500,18 +25500,18 @@
         </is>
       </c>
       <c r="F7" s="47" t="n">
-        <v>38.33</v>
+        <v>39.56</v>
       </c>
       <c r="G7" s="45" t="inlineStr">
         <is>
-          <t>10/19</t>
+          <t>10/20</t>
         </is>
       </c>
       <c r="H7" s="54" t="n">
-        <v>-4.15</v>
-      </c>
-      <c r="I7" s="48" t="n">
-        <v>-0.0977</v>
+        <v>1.23</v>
+      </c>
+      <c r="I7" s="49" t="n">
+        <v>0.0321</v>
       </c>
       <c r="J7" s="49" t="n">
         <v>0.05804878</v>
@@ -25574,18 +25574,18 @@
         </is>
       </c>
       <c r="F8" s="43" t="n">
-        <v>100.6</v>
+        <v>103.45</v>
       </c>
       <c r="G8" s="41" t="inlineStr">
         <is>
-          <t>10/19</t>
+          <t>10/20</t>
         </is>
       </c>
       <c r="H8" s="52" t="n">
-        <v>-7</v>
+        <v>-1.95</v>
       </c>
       <c r="I8" s="50" t="n">
-        <v>-0.06509999999999999</v>
+        <v>-0.0185</v>
       </c>
       <c r="J8" s="44" t="n">
         <v>0.00911528</v>
@@ -25644,18 +25644,18 @@
         </is>
       </c>
       <c r="F9" s="47" t="n">
-        <v>28.02</v>
+        <v>27.98</v>
       </c>
       <c r="G9" s="45" t="inlineStr">
         <is>
-          <t>10/19</t>
-        </is>
-      </c>
-      <c r="H9" s="56" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="I9" s="49" t="n">
-        <v>0.0018</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H9" s="55" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="I9" s="48" t="n">
+        <v>-0.0014</v>
       </c>
       <c r="J9" s="49" t="n">
         <v>0.05632139</v>
@@ -25718,18 +25718,18 @@
         </is>
       </c>
       <c r="F10" s="43" t="n">
-        <v>28.56</v>
+        <v>25.76</v>
       </c>
       <c r="G10" s="41" t="inlineStr">
         <is>
-          <t>10/19</t>
-        </is>
-      </c>
-      <c r="H10" s="55" t="n">
-        <v>2.74</v>
-      </c>
-      <c r="I10" s="44" t="n">
-        <v>0.1061</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H10" s="52" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="I10" s="50" t="n">
+        <v>-0.098</v>
       </c>
       <c r="J10" s="50" t="n">
         <v>-0.09624573</v>
@@ -25788,18 +25788,18 @@
         </is>
       </c>
       <c r="F11" s="47" t="n">
-        <v>53.15</v>
+        <v>49.11</v>
       </c>
       <c r="G11" s="45" t="inlineStr">
         <is>
-          <t>10/19</t>
-        </is>
-      </c>
-      <c r="H11" s="56" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="I11" s="49" t="n">
-        <v>0.063</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H11" s="55" t="n">
+        <v>-4.04</v>
+      </c>
+      <c r="I11" s="48" t="n">
+        <v>-0.076</v>
       </c>
       <c r="J11" s="49" t="n">
         <v>0.04219119</v>
@@ -25858,18 +25858,18 @@
         </is>
       </c>
       <c r="F12" s="43" t="n">
-        <v>108.3</v>
+        <v>96</v>
       </c>
       <c r="G12" s="41" t="inlineStr">
         <is>
-          <t>10/19</t>
-        </is>
-      </c>
-      <c r="H12" s="55" t="n">
-        <v>9.85</v>
-      </c>
-      <c r="I12" s="44" t="n">
-        <v>0.1001</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H12" s="52" t="n">
+        <v>-12.3</v>
+      </c>
+      <c r="I12" s="50" t="n">
+        <v>-0.1136</v>
       </c>
       <c r="J12" s="50" t="n">
         <v>-0.04014465</v>
@@ -25928,18 +25928,18 @@
         </is>
       </c>
       <c r="F13" s="47" t="n">
-        <v>87.5</v>
+        <v>81</v>
       </c>
       <c r="G13" s="45" t="inlineStr">
         <is>
-          <t>10/19</t>
-        </is>
-      </c>
-      <c r="H13" s="56" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="I13" s="49" t="n">
-        <v>0.0423</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H13" s="55" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="I13" s="48" t="n">
+        <v>-0.07429999999999999</v>
       </c>
       <c r="J13" s="48" t="n">
         <v>-0.11655405</v>
@@ -25998,18 +25998,18 @@
         </is>
       </c>
       <c r="F14" s="43" t="n">
-        <v>66.2</v>
+        <v>63.7</v>
       </c>
       <c r="G14" s="41" t="inlineStr">
         <is>
-          <t>10/19</t>
-        </is>
-      </c>
-      <c r="H14" s="55" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="I14" s="44" t="n">
-        <v>0.0192</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H14" s="52" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="I14" s="50" t="n">
+        <v>-0.0378</v>
       </c>
       <c r="J14" s="44" t="n">
         <v>0.03063547</v>
@@ -26068,18 +26068,18 @@
         </is>
       </c>
       <c r="F15" s="47" t="n">
-        <v>46.6</v>
+        <v>43.4</v>
       </c>
       <c r="G15" s="45" t="inlineStr">
         <is>
-          <t>10/19</t>
-        </is>
-      </c>
-      <c r="H15" s="56" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="I15" s="49" t="n">
-        <v>0.0507</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H15" s="55" t="n">
+        <v>-3.2</v>
+      </c>
+      <c r="I15" s="48" t="n">
+        <v>-0.0687</v>
       </c>
       <c r="J15" s="48" t="n">
         <v>-0.04295893000000001</v>
@@ -26138,18 +26138,18 @@
         </is>
       </c>
       <c r="F16" s="43" t="n">
-        <v>14.4</v>
+        <v>14.61</v>
       </c>
       <c r="G16" s="41" t="inlineStr">
         <is>
-          <t>10/19</t>
+          <t>10/20</t>
         </is>
       </c>
       <c r="H16" s="52" t="n">
-        <v>-0.61</v>
+        <v>-0.24</v>
       </c>
       <c r="I16" s="50" t="n">
-        <v>-0.0406</v>
+        <v>-0.0162</v>
       </c>
       <c r="J16" s="53" t="inlineStr"/>
       <c r="K16" s="53" t="inlineStr"/>
@@ -26409,7 +26409,7 @@
           <t>10/16</t>
         </is>
       </c>
-      <c r="H3" s="54" t="n">
+      <c r="H3" s="55" t="n">
         <v>-0.0844</v>
       </c>
       <c r="I3" s="48" t="n">
@@ -26483,7 +26483,7 @@
           <t>10/16</t>
         </is>
       </c>
-      <c r="H4" s="55" t="n">
+      <c r="H4" s="56" t="n">
         <v>0.0009</v>
       </c>
       <c r="I4" s="44" t="n">
@@ -26557,7 +26557,7 @@
           <t>10/16</t>
         </is>
       </c>
-      <c r="H5" s="54" t="n">
+      <c r="H5" s="55" t="n">
         <v>-0.0069</v>
       </c>
       <c r="I5" s="48" t="n">
@@ -26705,7 +26705,7 @@
           <t>10/16</t>
         </is>
       </c>
-      <c r="H7" s="54" t="n">
+      <c r="H7" s="55" t="n">
         <v>-0.007</v>
       </c>
       <c r="I7" s="48" t="n">
@@ -26779,7 +26779,7 @@
           <t>10/16</t>
         </is>
       </c>
-      <c r="H8" s="55" t="n">
+      <c r="H8" s="56" t="n">
         <v>0.0009</v>
       </c>
       <c r="I8" s="44" t="n">
@@ -26853,7 +26853,7 @@
           <t>10/19</t>
         </is>
       </c>
-      <c r="H9" s="54" t="n">
+      <c r="H9" s="55" t="n">
         <v>-0.66</v>
       </c>
       <c r="I9" s="48" t="n">
@@ -27001,7 +27001,7 @@
           <t>10/19</t>
         </is>
       </c>
-      <c r="H11" s="54" t="n">
+      <c r="H11" s="55" t="n">
         <v>-0.85</v>
       </c>
       <c r="I11" s="48" t="n">

</xml_diff>

<commit_message>
chore: 自動更新最新基金與ETF數據 (2026-10-21 16:13:02)
</commit_message>
<xml_diff>
--- a/國泰投信_人氣ETF與熱門基金分析.xlsx
+++ b/國泰投信_人氣ETF與熱門基金分析.xlsx
@@ -362,7 +362,7 @@
     <xf numFmtId="10" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -371,10 +371,10 @@
     <xf numFmtId="4" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1725,7 +1725,7 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>國泰台灣科技龍頭 (00881) (台積電佔比: 39.86% (科技純度: 95.26%))</t>
+          <t>國泰台灣科技龍頭 (00881) (台積電佔比: 40.31% (科技純度: 95.33%))</t>
         </is>
       </c>
     </row>
@@ -13097,22 +13097,22 @@
         </is>
       </c>
       <c r="D5" s="23" t="n">
-        <v>0.08710000000000001</v>
+        <v>0.08900000000000001</v>
       </c>
       <c r="E5" s="23" t="n">
-        <v>0.6758999999999999</v>
+        <v>0.6923000000000004</v>
       </c>
       <c r="F5" s="23" t="n">
-        <v>0.7629999999999998</v>
+        <v>0.7813000000000003</v>
       </c>
       <c r="G5" s="23" t="n">
-        <v>0.032</v>
+        <v>0.0319</v>
       </c>
       <c r="H5" s="23" t="n">
         <v>0.118</v>
       </c>
       <c r="I5" s="21" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="J5" s="21" t="inlineStr">
         <is>
@@ -13121,7 +13121,7 @@
       </c>
       <c r="K5" s="21" t="inlineStr">
         <is>
-          <t>台積電(8.71%), 聯發科(6.16%), 台光電(4.28%)</t>
+          <t>台積電(8.9%), 聯發科(6.92%), 南亞(4.34%)</t>
         </is>
       </c>
     </row>
@@ -13145,16 +13145,16 @@
         <v>0</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>0.5079</v>
+        <v>0.5125000000000001</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.5079</v>
+        <v>0.5125000000000001</v>
       </c>
       <c r="G6" s="29" t="n">
-        <v>0.3598000000000001</v>
+        <v>0.3545</v>
       </c>
       <c r="H6" s="29" t="n">
-        <v>0.1039</v>
+        <v>0.1038</v>
       </c>
       <c r="I6" s="27" t="n">
         <v>0</v>
@@ -13166,7 +13166,7 @@
       </c>
       <c r="K6" s="27" t="inlineStr">
         <is>
-          <t>中信金(10.22%), 廣達(8.51%), 國泰金(6.54%)</t>
+          <t>中信金(10.07%), 廣達(8.75%), 國泰金(6.34%)</t>
         </is>
       </c>
     </row>
@@ -13277,22 +13277,22 @@
         </is>
       </c>
       <c r="D9" s="23" t="n">
-        <v>0.3986</v>
+        <v>0.4031</v>
       </c>
       <c r="E9" s="23" t="n">
-        <v>0.5539999999999999</v>
+        <v>0.5502000000000001</v>
       </c>
       <c r="F9" s="23" t="n">
-        <v>0.9525999999999999</v>
+        <v>0.9533000000000001</v>
       </c>
       <c r="G9" s="25" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="23" t="n">
-        <v>0.0213</v>
+        <v>0.02039999999999999</v>
       </c>
       <c r="I9" s="21" t="n">
-        <v>0.004</v>
+        <v>0.0063</v>
       </c>
       <c r="J9" s="21" t="inlineStr">
         <is>
@@ -13301,7 +13301,7 @@
       </c>
       <c r="K9" s="21" t="inlineStr">
         <is>
-          <t>台積電(39.86%), 聯發科(10.08%), 台達電(5.47%)</t>
+          <t>台積電(40.31%), 聯發科(9.74%), 台達電(5.25%)</t>
         </is>
       </c>
     </row>
@@ -13322,19 +13322,19 @@
         </is>
       </c>
       <c r="D10" s="29" t="n">
-        <v>0.3937</v>
+        <v>0.3959</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.4217000000000001</v>
+        <v>0.4213999999999999</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>0.8154</v>
+        <v>0.8172999999999999</v>
       </c>
       <c r="G10" s="29" t="n">
-        <v>0.1362</v>
+        <v>0.1345</v>
       </c>
       <c r="H10" s="29" t="n">
-        <v>0.0348</v>
+        <v>0.0346</v>
       </c>
       <c r="I10" s="27" t="n">
         <v>0</v>
@@ -13346,7 +13346,7 @@
       </c>
       <c r="K10" s="27" t="inlineStr">
         <is>
-          <t>台積電(39.37%), 聯發科(6.64%), 台達電(3.8%)</t>
+          <t>台積電(39.59%), 聯發科(6.64%), 台達電(3.77%)</t>
         </is>
       </c>
     </row>
@@ -13427,7 +13427,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="27" t="n">
-        <v>0.9995000000000001</v>
+        <v>0.9994</v>
       </c>
       <c r="J12" s="27" t="inlineStr">
         <is>
@@ -13436,7 +13436,7 @@
       </c>
       <c r="K12" s="27" t="inlineStr">
         <is>
-          <t>Apple Inc.(17.36%), Microsoft Corp(14.2%), AMAZON.COM INC(9.31%)</t>
+          <t>Apple Inc.(17.22%), Microsoft Corp(14.19%), AMAZON.COM INC(9.33%)</t>
         </is>
       </c>
     </row>
@@ -13472,7 +13472,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="21" t="n">
-        <v>0.9726999999999997</v>
+        <v>0.9728000000000001</v>
       </c>
       <c r="J13" s="21" t="inlineStr">
         <is>
@@ -13481,7 +13481,7 @@
       </c>
       <c r="K13" s="21" t="inlineStr">
         <is>
-          <t>貴州茅台(8.74%), 寧德時代(6.41%), 招商銀行(4.6%)</t>
+          <t>貴州茅台(8.81%), 寧德時代(6.04%), 招商銀行(4.63%)</t>
         </is>
       </c>
     </row>
@@ -13502,22 +13502,22 @@
         </is>
       </c>
       <c r="D14" s="29" t="n">
-        <v>0.2261</v>
+        <v>0.2283</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.4155</v>
+        <v>0.4168000000000001</v>
       </c>
       <c r="F14" s="29" t="n">
-        <v>0.6415999999999999</v>
+        <v>0.6451000000000002</v>
       </c>
       <c r="G14" s="31" t="n">
         <v>0</v>
       </c>
       <c r="H14" s="29" t="n">
-        <v>0.009399999999999999</v>
+        <v>0.0098</v>
       </c>
       <c r="I14" s="27" t="n">
-        <v>0.3295999999999999</v>
+        <v>0.3254</v>
       </c>
       <c r="J14" s="27" t="inlineStr">
         <is>
@@ -13526,7 +13526,7 @@
       </c>
       <c r="K14" s="27" t="inlineStr">
         <is>
-          <t>台積電(22.61%), Samsung Electron Rg(15.03%), SK Hynix Inc(11.28%)</t>
+          <t>台積電(22.83%), Samsung Electron Rg(14.91%), SK Hynix Inc(11.05%)</t>
         </is>
       </c>
     </row>
@@ -13571,7 +13571,7 @@
       </c>
       <c r="K15" s="21" t="inlineStr">
         <is>
-          <t>NVIDIA CORPORATION(12.04%), BROADCOM INC(9.22%), Micron Technology Inc(7.71%)</t>
+          <t>NVIDIA CORPORATION(12.04%), BROADCOM INC(9.24%), Micron Technology Inc(7.65%)</t>
         </is>
       </c>
     </row>
@@ -13607,7 +13607,7 @@
         <v>0</v>
       </c>
       <c r="I16" s="27" t="n">
-        <v>0.9869000000000027</v>
+        <v>0.9874000000000028</v>
       </c>
       <c r="J16" s="27" t="inlineStr">
         <is>
@@ -13616,7 +13616,7 @@
       </c>
       <c r="K16" s="27" t="inlineStr">
         <is>
-          <t>Apple Inc.(9.2%), Microsoft Corp(9.18%), NVIDIA CORPORATION(8.21%)</t>
+          <t>Microsoft Corp(9.18%), Apple Inc.(9.13%), NVIDIA CORPORATION(8.21%)</t>
         </is>
       </c>
     </row>
@@ -13640,10 +13640,10 @@
         <v>0</v>
       </c>
       <c r="E17" s="23" t="n">
-        <v>0.0341</v>
+        <v>0.0335</v>
       </c>
       <c r="F17" s="23" t="n">
-        <v>0.0341</v>
+        <v>0.0335</v>
       </c>
       <c r="G17" s="25" t="n">
         <v>0</v>
@@ -13652,7 +13652,7 @@
         <v>0</v>
       </c>
       <c r="I17" s="21" t="n">
-        <v>0.9521999999999999</v>
+        <v>0.9196999999999997</v>
       </c>
       <c r="J17" s="21" t="inlineStr">
         <is>
@@ -13661,7 +13661,7 @@
       </c>
       <c r="K17" s="21" t="inlineStr">
         <is>
-          <t>ADV MICRO DEVICES(25.97%), NVIDIA CORPORATION(14.43%), TESLA, INC.(12.32%)</t>
+          <t>ADV MICRO DEVICES(25.96%), NVIDIA CORPORATION(14.47%), TESLA, INC.(12.58%)</t>
         </is>
       </c>
     </row>
@@ -14249,11 +14249,11 @@
         </is>
       </c>
       <c r="H33" s="23" t="n">
-        <v>0.08710000000000001</v>
+        <v>0.08900000000000001</v>
       </c>
       <c r="I33" s="21" t="inlineStr">
         <is>
-          <t>1,094,000</t>
+          <t>1,131,000</t>
         </is>
       </c>
     </row>
@@ -14292,11 +14292,11 @@
         </is>
       </c>
       <c r="H34" s="29" t="n">
-        <v>0.0616</v>
+        <v>0.0692</v>
       </c>
       <c r="I34" s="27" t="inlineStr">
         <is>
-          <t>445,000</t>
+          <t>514,000</t>
         </is>
       </c>
     </row>
@@ -14321,25 +14321,25 @@
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>2383</t>
+          <t>1303</t>
         </is>
       </c>
       <c r="F35" s="21" t="inlineStr">
         <is>
-          <t>台光電</t>
+          <t>南亞</t>
         </is>
       </c>
       <c r="G35" s="21" t="inlineStr">
         <is>
-          <t>科技電子</t>
+          <t>傳統產業</t>
         </is>
       </c>
       <c r="H35" s="25" t="n">
-        <v>0.0428</v>
+        <v>0.0434</v>
       </c>
       <c r="I35" s="21" t="inlineStr">
         <is>
-          <t>254,000</t>
+          <t>4,167,000</t>
         </is>
       </c>
     </row>
@@ -14364,25 +14364,25 @@
       </c>
       <c r="E36" s="26" t="inlineStr">
         <is>
-          <t>1303</t>
+          <t>2383</t>
         </is>
       </c>
       <c r="F36" s="27" t="inlineStr">
         <is>
-          <t>南亞</t>
+          <t>台光電</t>
         </is>
       </c>
       <c r="G36" s="27" t="inlineStr">
         <is>
-          <t>傳統產業</t>
+          <t>科技電子</t>
         </is>
       </c>
       <c r="H36" s="31" t="n">
-        <v>0.0416</v>
+        <v>0.0412</v>
       </c>
       <c r="I36" s="27" t="inlineStr">
         <is>
-          <t>4,167,000</t>
+          <t>254,000</t>
         </is>
       </c>
     </row>
@@ -14421,7 +14421,7 @@
         </is>
       </c>
       <c r="H37" s="25" t="n">
-        <v>0.0394</v>
+        <v>0.0383</v>
       </c>
       <c r="I37" s="21" t="inlineStr">
         <is>
@@ -14450,25 +14450,25 @@
       </c>
       <c r="E38" s="26" t="inlineStr">
         <is>
-          <t>3017</t>
+          <t>2059</t>
         </is>
       </c>
       <c r="F38" s="27" t="inlineStr">
         <is>
-          <t>奇鋐</t>
+          <t>川湖</t>
         </is>
       </c>
       <c r="G38" s="27" t="inlineStr">
         <is>
-          <t>科技電子</t>
+          <t>傳統產業</t>
         </is>
       </c>
       <c r="H38" s="31" t="n">
-        <v>0.0359</v>
+        <v>0.0367</v>
       </c>
       <c r="I38" s="27" t="inlineStr">
         <is>
-          <t>329,000</t>
+          <t>112,000</t>
         </is>
       </c>
     </row>
@@ -14493,12 +14493,12 @@
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>3653</t>
+          <t>3017</t>
         </is>
       </c>
       <c r="F39" s="21" t="inlineStr">
         <is>
-          <t>健策</t>
+          <t>奇鋐</t>
         </is>
       </c>
       <c r="G39" s="21" t="inlineStr">
@@ -14507,11 +14507,11 @@
         </is>
       </c>
       <c r="H39" s="25" t="n">
-        <v>0.0332</v>
+        <v>0.0346</v>
       </c>
       <c r="I39" s="21" t="inlineStr">
         <is>
-          <t>154,000</t>
+          <t>329,000</t>
         </is>
       </c>
     </row>
@@ -14536,12 +14536,12 @@
       </c>
       <c r="E40" s="26" t="inlineStr">
         <is>
-          <t>6223</t>
+          <t>3653</t>
         </is>
       </c>
       <c r="F40" s="27" t="inlineStr">
         <is>
-          <t>旺矽</t>
+          <t>健策</t>
         </is>
       </c>
       <c r="G40" s="27" t="inlineStr">
@@ -14550,11 +14550,11 @@
         </is>
       </c>
       <c r="H40" s="31" t="n">
-        <v>0.0312</v>
+        <v>0.0327</v>
       </c>
       <c r="I40" s="27" t="inlineStr">
         <is>
-          <t>181,000</t>
+          <t>154,000</t>
         </is>
       </c>
     </row>
@@ -14593,7 +14593,7 @@
         </is>
       </c>
       <c r="H41" s="25" t="n">
-        <v>0.031</v>
+        <v>0.0307</v>
       </c>
       <c r="I41" s="21" t="inlineStr">
         <is>
@@ -14622,12 +14622,12 @@
       </c>
       <c r="E42" s="26" t="inlineStr">
         <is>
-          <t>2368</t>
+          <t>6223</t>
         </is>
       </c>
       <c r="F42" s="27" t="inlineStr">
         <is>
-          <t>金像電</t>
+          <t>旺矽</t>
         </is>
       </c>
       <c r="G42" s="27" t="inlineStr">
@@ -14636,11 +14636,11 @@
         </is>
       </c>
       <c r="H42" s="31" t="n">
-        <v>0.0302</v>
+        <v>0.0295</v>
       </c>
       <c r="I42" s="27" t="inlineStr">
         <is>
-          <t>734,000</t>
+          <t>181,000</t>
         </is>
       </c>
     </row>
@@ -14679,7 +14679,7 @@
         </is>
       </c>
       <c r="H43" s="23" t="n">
-        <v>0.1022</v>
+        <v>0.1007</v>
       </c>
       <c r="I43" s="21" t="inlineStr">
         <is>
@@ -14722,7 +14722,7 @@
         </is>
       </c>
       <c r="H44" s="29" t="n">
-        <v>0.0851</v>
+        <v>0.08749999999999999</v>
       </c>
       <c r="I44" s="27" t="inlineStr">
         <is>
@@ -14765,7 +14765,7 @@
         </is>
       </c>
       <c r="H45" s="23" t="n">
-        <v>0.0654</v>
+        <v>0.0634</v>
       </c>
       <c r="I45" s="21" t="inlineStr">
         <is>
@@ -14808,7 +14808,7 @@
         </is>
       </c>
       <c r="H46" s="29" t="n">
-        <v>0.0576</v>
+        <v>0.05889999999999999</v>
       </c>
       <c r="I46" s="27" t="inlineStr">
         <is>
@@ -14894,7 +14894,7 @@
         </is>
       </c>
       <c r="H48" s="31" t="n">
-        <v>0.0385</v>
+        <v>0.03759999999999999</v>
       </c>
       <c r="I48" s="27" t="inlineStr">
         <is>
@@ -14937,7 +14937,7 @@
         </is>
       </c>
       <c r="H49" s="25" t="n">
-        <v>0.03759999999999999</v>
+        <v>0.0367</v>
       </c>
       <c r="I49" s="21" t="inlineStr">
         <is>
@@ -14980,7 +14980,7 @@
         </is>
       </c>
       <c r="H50" s="31" t="n">
-        <v>0.0329</v>
+        <v>0.0328</v>
       </c>
       <c r="I50" s="27" t="inlineStr">
         <is>
@@ -15009,12 +15009,12 @@
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>2454</t>
+          <t>2379</t>
         </is>
       </c>
       <c r="F51" s="21" t="inlineStr">
         <is>
-          <t>聯發科</t>
+          <t>瑞昱</t>
         </is>
       </c>
       <c r="G51" s="21" t="inlineStr">
@@ -15023,11 +15023,11 @@
         </is>
       </c>
       <c r="H51" s="25" t="n">
-        <v>0.0327</v>
+        <v>0.0326</v>
       </c>
       <c r="I51" s="21" t="inlineStr">
         <is>
-          <t>5,179,000</t>
+          <t>27,834,000</t>
         </is>
       </c>
     </row>
@@ -15052,12 +15052,12 @@
       </c>
       <c r="E52" s="26" t="inlineStr">
         <is>
-          <t>2379</t>
+          <t>2454</t>
         </is>
       </c>
       <c r="F52" s="27" t="inlineStr">
         <is>
-          <t>瑞昱</t>
+          <t>聯發科</t>
         </is>
       </c>
       <c r="G52" s="27" t="inlineStr">
@@ -15070,7 +15070,7 @@
       </c>
       <c r="I52" s="27" t="inlineStr">
         <is>
-          <t>27,834,000</t>
+          <t>5,179,000</t>
         </is>
       </c>
     </row>
@@ -15809,11 +15809,11 @@
         </is>
       </c>
       <c r="H73" s="23" t="n">
-        <v>0.3986</v>
+        <v>0.4031</v>
       </c>
       <c r="I73" s="21" t="inlineStr">
         <is>
-          <t>24,485,000</t>
+          <t>24,613,000</t>
         </is>
       </c>
     </row>
@@ -15852,11 +15852,11 @@
         </is>
       </c>
       <c r="H74" s="29" t="n">
-        <v>0.1008</v>
+        <v>0.0974</v>
       </c>
       <c r="I74" s="27" t="inlineStr">
         <is>
-          <t>3,562,000</t>
+          <t>3,446,000</t>
         </is>
       </c>
     </row>
@@ -15895,11 +15895,11 @@
         </is>
       </c>
       <c r="H75" s="23" t="n">
-        <v>0.0547</v>
+        <v>0.0525</v>
       </c>
       <c r="I75" s="21" t="inlineStr">
         <is>
-          <t>4,958,000</t>
+          <t>4,802,000</t>
         </is>
       </c>
     </row>
@@ -15938,7 +15938,7 @@
         </is>
       </c>
       <c r="H76" s="31" t="n">
-        <v>0.0461</v>
+        <v>0.0471</v>
       </c>
       <c r="I76" s="27" t="inlineStr">
         <is>
@@ -15967,12 +15967,12 @@
       </c>
       <c r="E77" s="20" t="inlineStr">
         <is>
-          <t>3037</t>
+          <t>2383</t>
         </is>
       </c>
       <c r="F77" s="21" t="inlineStr">
         <is>
-          <t>欣興</t>
+          <t>台光電</t>
         </is>
       </c>
       <c r="G77" s="21" t="inlineStr">
@@ -15981,11 +15981,11 @@
         </is>
       </c>
       <c r="H77" s="25" t="n">
-        <v>0.0292</v>
+        <v>0.0262</v>
       </c>
       <c r="I77" s="21" t="inlineStr">
         <is>
-          <t>3,872,871</t>
+          <t>777,000</t>
         </is>
       </c>
     </row>
@@ -16010,12 +16010,12 @@
       </c>
       <c r="E78" s="26" t="inlineStr">
         <is>
-          <t>2303</t>
+          <t>3037</t>
         </is>
       </c>
       <c r="F78" s="27" t="inlineStr">
         <is>
-          <t>聯電</t>
+          <t>欣興</t>
         </is>
       </c>
       <c r="G78" s="27" t="inlineStr">
@@ -16024,11 +16024,11 @@
         </is>
       </c>
       <c r="H78" s="31" t="n">
-        <v>0.0265</v>
+        <v>0.026</v>
       </c>
       <c r="I78" s="27" t="inlineStr">
         <is>
-          <t>29,935,000</t>
+          <t>3,624,871</t>
         </is>
       </c>
     </row>
@@ -16053,12 +16053,12 @@
       </c>
       <c r="E79" s="20" t="inlineStr">
         <is>
-          <t>2383</t>
+          <t>3017</t>
         </is>
       </c>
       <c r="F79" s="21" t="inlineStr">
         <is>
-          <t>台光電</t>
+          <t>奇鋐</t>
         </is>
       </c>
       <c r="G79" s="21" t="inlineStr">
@@ -16067,11 +16067,11 @@
         </is>
       </c>
       <c r="H79" s="25" t="n">
-        <v>0.0265</v>
+        <v>0.0241</v>
       </c>
       <c r="I79" s="21" t="inlineStr">
         <is>
-          <t>768,000</t>
+          <t>1,066,000</t>
         </is>
       </c>
     </row>
@@ -16096,12 +16096,12 @@
       </c>
       <c r="E80" s="26" t="inlineStr">
         <is>
-          <t>3017</t>
+          <t>2303</t>
         </is>
       </c>
       <c r="F80" s="27" t="inlineStr">
         <is>
-          <t>奇鋐</t>
+          <t>聯電</t>
         </is>
       </c>
       <c r="G80" s="27" t="inlineStr">
@@ -16110,11 +16110,11 @@
         </is>
       </c>
       <c r="H80" s="31" t="n">
-        <v>0.0232</v>
+        <v>0.024</v>
       </c>
       <c r="I80" s="27" t="inlineStr">
         <is>
-          <t>1,040,000</t>
+          <t>27,765,000</t>
         </is>
       </c>
     </row>
@@ -16153,11 +16153,11 @@
         </is>
       </c>
       <c r="H81" s="25" t="n">
-        <v>0.0224</v>
+        <v>0.0231</v>
       </c>
       <c r="I81" s="21" t="inlineStr">
         <is>
-          <t>1,663,000</t>
+          <t>1,719,000</t>
         </is>
       </c>
     </row>
@@ -16182,25 +16182,25 @@
       </c>
       <c r="E82" s="26" t="inlineStr">
         <is>
-          <t>2059</t>
+          <t>2382</t>
         </is>
       </c>
       <c r="F82" s="27" t="inlineStr">
         <is>
-          <t>川湖</t>
+          <t>廣達</t>
         </is>
       </c>
       <c r="G82" s="27" t="inlineStr">
         <is>
-          <t>傳統產業</t>
+          <t>科技電子</t>
         </is>
       </c>
       <c r="H82" s="31" t="n">
-        <v>0.021</v>
+        <v>0.0214</v>
       </c>
       <c r="I82" s="27" t="inlineStr">
         <is>
-          <t>315,000</t>
+          <t>9,807,000</t>
         </is>
       </c>
     </row>
@@ -16239,11 +16239,11 @@
         </is>
       </c>
       <c r="H83" s="23" t="n">
-        <v>0.3937</v>
+        <v>0.3959</v>
       </c>
       <c r="I83" s="21" t="inlineStr">
         <is>
-          <t>14,811,446</t>
+          <t>14,827,736</t>
         </is>
       </c>
     </row>
@@ -16286,7 +16286,7 @@
       </c>
       <c r="I84" s="27" t="inlineStr">
         <is>
-          <t>1,438,711</t>
+          <t>1,440,321</t>
         </is>
       </c>
     </row>
@@ -16325,11 +16325,11 @@
         </is>
       </c>
       <c r="H85" s="25" t="n">
-        <v>0.038</v>
+        <v>0.0377</v>
       </c>
       <c r="I85" s="21" t="inlineStr">
         <is>
-          <t>2,110,739</t>
+          <t>2,113,099</t>
         </is>
       </c>
     </row>
@@ -16368,11 +16368,11 @@
         </is>
       </c>
       <c r="H86" s="31" t="n">
-        <v>0.0325</v>
+        <v>0.0332</v>
       </c>
       <c r="I86" s="27" t="inlineStr">
         <is>
-          <t>12,360,359</t>
+          <t>12,374,194</t>
         </is>
       </c>
     </row>
@@ -16411,11 +16411,11 @@
         </is>
       </c>
       <c r="H87" s="25" t="n">
-        <v>0.0299</v>
+        <v>0.0298</v>
       </c>
       <c r="I87" s="21" t="inlineStr">
         <is>
-          <t>4,059,924</t>
+          <t>4,064,469</t>
         </is>
       </c>
     </row>
@@ -16454,11 +16454,11 @@
         </is>
       </c>
       <c r="H88" s="31" t="n">
-        <v>0.0213</v>
+        <v>0.0208</v>
       </c>
       <c r="I88" s="27" t="inlineStr">
         <is>
-          <t>378,359</t>
+          <t>378,779</t>
         </is>
       </c>
     </row>
@@ -16497,11 +16497,11 @@
         </is>
       </c>
       <c r="H89" s="25" t="n">
-        <v>0.0208</v>
+        <v>0.0203</v>
       </c>
       <c r="I89" s="21" t="inlineStr">
         <is>
-          <t>14,404,513</t>
+          <t>14,420,638</t>
         </is>
       </c>
     </row>
@@ -16540,11 +16540,11 @@
         </is>
       </c>
       <c r="H90" s="31" t="n">
-        <v>0.0184</v>
+        <v>0.0181</v>
       </c>
       <c r="I90" s="27" t="inlineStr">
         <is>
-          <t>10,595,170</t>
+          <t>10,607,045</t>
         </is>
       </c>
     </row>
@@ -16583,11 +16583,11 @@
         </is>
       </c>
       <c r="H91" s="25" t="n">
-        <v>0.0176</v>
+        <v>0.0173</v>
       </c>
       <c r="I91" s="21" t="inlineStr">
         <is>
-          <t>5,265,178</t>
+          <t>5,271,073</t>
         </is>
       </c>
     </row>
@@ -16626,11 +16626,11 @@
         </is>
       </c>
       <c r="H92" s="31" t="n">
-        <v>0.017</v>
+        <v>0.0172</v>
       </c>
       <c r="I92" s="27" t="inlineStr">
         <is>
-          <t>465,334</t>
+          <t>465,854</t>
         </is>
       </c>
     </row>
@@ -16669,7 +16669,7 @@
         </is>
       </c>
       <c r="H93" s="23" t="n">
-        <v>0.1736</v>
+        <v>0.1722</v>
       </c>
       <c r="I93" s="21" t="inlineStr">
         <is>
@@ -16712,7 +16712,7 @@
         </is>
       </c>
       <c r="H94" s="29" t="n">
-        <v>0.142</v>
+        <v>0.1419</v>
       </c>
       <c r="I94" s="27" t="inlineStr">
         <is>
@@ -16755,7 +16755,7 @@
         </is>
       </c>
       <c r="H95" s="23" t="n">
-        <v>0.0931</v>
+        <v>0.09329999999999999</v>
       </c>
       <c r="I95" s="21" t="inlineStr">
         <is>
@@ -16798,7 +16798,7 @@
         </is>
       </c>
       <c r="H96" s="29" t="n">
-        <v>0.0728</v>
+        <v>0.0721</v>
       </c>
       <c r="I96" s="27" t="inlineStr">
         <is>
@@ -16841,7 +16841,7 @@
         </is>
       </c>
       <c r="H97" s="23" t="n">
-        <v>0.0562</v>
+        <v>0.0554</v>
       </c>
       <c r="I97" s="21" t="inlineStr">
         <is>
@@ -16884,7 +16884,7 @@
         </is>
       </c>
       <c r="H98" s="31" t="n">
-        <v>0.0378</v>
+        <v>0.0384</v>
       </c>
       <c r="I98" s="27" t="inlineStr">
         <is>
@@ -16927,7 +16927,7 @@
         </is>
       </c>
       <c r="H99" s="25" t="n">
-        <v>0.0326</v>
+        <v>0.0329</v>
       </c>
       <c r="I99" s="21" t="inlineStr">
         <is>
@@ -16970,7 +16970,7 @@
         </is>
       </c>
       <c r="H100" s="31" t="n">
-        <v>0.0302</v>
+        <v>0.0295</v>
       </c>
       <c r="I100" s="27" t="inlineStr">
         <is>
@@ -17013,7 +17013,7 @@
         </is>
       </c>
       <c r="H101" s="25" t="n">
-        <v>0.0246</v>
+        <v>0.0249</v>
       </c>
       <c r="I101" s="21" t="inlineStr">
         <is>
@@ -17056,7 +17056,7 @@
         </is>
       </c>
       <c r="H102" s="31" t="n">
-        <v>0.0189</v>
+        <v>0.0188</v>
       </c>
       <c r="I102" s="27" t="inlineStr">
         <is>
@@ -17099,11 +17099,11 @@
         </is>
       </c>
       <c r="H103" s="23" t="n">
-        <v>0.08740000000000001</v>
+        <v>0.08810000000000001</v>
       </c>
       <c r="I103" s="21" t="inlineStr">
         <is>
-          <t>33,119</t>
+          <t>32,919</t>
         </is>
       </c>
     </row>
@@ -17142,11 +17142,11 @@
         </is>
       </c>
       <c r="H104" s="29" t="n">
-        <v>0.0641</v>
+        <v>0.0604</v>
       </c>
       <c r="I104" s="27" t="inlineStr">
         <is>
-          <t>116,540</t>
+          <t>115,940</t>
         </is>
       </c>
     </row>
@@ -17185,11 +17185,11 @@
         </is>
       </c>
       <c r="H105" s="25" t="n">
-        <v>0.046</v>
+        <v>0.0463</v>
       </c>
       <c r="I105" s="21" t="inlineStr">
         <is>
-          <t>545,156</t>
+          <t>542,356</t>
         </is>
       </c>
     </row>
@@ -17214,12 +17214,12 @@
       </c>
       <c r="E106" s="26" t="inlineStr">
         <is>
-          <t>300308.CH</t>
+          <t>600900.CH</t>
         </is>
       </c>
       <c r="F106" s="27" t="inlineStr">
         <is>
-          <t>Zhongji Innolight (A) (SC SZ)</t>
+          <t>長江電力</t>
         </is>
       </c>
       <c r="G106" s="27" t="inlineStr">
@@ -17228,11 +17228,11 @@
         </is>
       </c>
       <c r="H106" s="31" t="n">
-        <v>0.0391</v>
+        <v>0.0384</v>
       </c>
       <c r="I106" s="27" t="inlineStr">
         <is>
-          <t>29,400</t>
+          <t>643,329</t>
         </is>
       </c>
     </row>
@@ -17257,12 +17257,12 @@
       </c>
       <c r="E107" s="20" t="inlineStr">
         <is>
-          <t>600900.CH</t>
+          <t>300308.CH</t>
         </is>
       </c>
       <c r="F107" s="21" t="inlineStr">
         <is>
-          <t>長江電力</t>
+          <t>Zhongji Innolight (A) (SC SZ)</t>
         </is>
       </c>
       <c r="G107" s="21" t="inlineStr">
@@ -17271,11 +17271,11 @@
         </is>
       </c>
       <c r="H107" s="25" t="n">
-        <v>0.0377</v>
+        <v>0.0383</v>
       </c>
       <c r="I107" s="21" t="inlineStr">
         <is>
-          <t>646,629</t>
+          <t>29,400</t>
         </is>
       </c>
     </row>
@@ -17300,12 +17300,12 @@
       </c>
       <c r="E108" s="26" t="inlineStr">
         <is>
-          <t>601398.CH</t>
+          <t>601288.CH</t>
         </is>
       </c>
       <c r="F108" s="27" t="inlineStr">
         <is>
-          <t>工商銀行</t>
+          <t>農業銀行</t>
         </is>
       </c>
       <c r="G108" s="27" t="inlineStr">
@@ -17314,11 +17314,11 @@
         </is>
       </c>
       <c r="H108" s="31" t="n">
-        <v>0.0338</v>
+        <v>0.0347</v>
       </c>
       <c r="I108" s="27" t="inlineStr">
         <is>
-          <t>2,008,327</t>
+          <t>2,332,700</t>
         </is>
       </c>
     </row>
@@ -17343,12 +17343,12 @@
       </c>
       <c r="E109" s="20" t="inlineStr">
         <is>
-          <t>601288.CH</t>
+          <t>601398.CH</t>
         </is>
       </c>
       <c r="F109" s="21" t="inlineStr">
         <is>
-          <t>農業銀行</t>
+          <t>工商銀行</t>
         </is>
       </c>
       <c r="G109" s="21" t="inlineStr">
@@ -17357,11 +17357,11 @@
         </is>
       </c>
       <c r="H109" s="25" t="n">
-        <v>0.0337</v>
+        <v>0.0345</v>
       </c>
       <c r="I109" s="21" t="inlineStr">
         <is>
-          <t>2,344,800</t>
+          <t>1,997,927</t>
         </is>
       </c>
     </row>
@@ -17400,11 +17400,11 @@
         </is>
       </c>
       <c r="H110" s="31" t="n">
-        <v>0.03240000000000001</v>
+        <v>0.0316</v>
       </c>
       <c r="I110" s="27" t="inlineStr">
         <is>
-          <t>544,469</t>
+          <t>541,669</t>
         </is>
       </c>
     </row>
@@ -17443,7 +17443,7 @@
         </is>
       </c>
       <c r="H111" s="25" t="n">
-        <v>0.0301</v>
+        <v>0.0307</v>
       </c>
       <c r="I111" s="21" t="inlineStr">
         <is>
@@ -17472,12 +17472,12 @@
       </c>
       <c r="E112" s="26" t="inlineStr">
         <is>
-          <t>601318.CH</t>
+          <t>601138.CH</t>
         </is>
       </c>
       <c r="F112" s="27" t="inlineStr">
         <is>
-          <t>中國平安</t>
+          <t>工業富聯</t>
         </is>
       </c>
       <c r="G112" s="27" t="inlineStr">
@@ -17486,11 +17486,11 @@
         </is>
       </c>
       <c r="H112" s="31" t="n">
-        <v>0.029</v>
+        <v>0.0296</v>
       </c>
       <c r="I112" s="27" t="inlineStr">
         <is>
-          <t>281,709</t>
+          <t>301,774</t>
         </is>
       </c>
     </row>
@@ -17529,7 +17529,7 @@
         </is>
       </c>
       <c r="H113" s="23" t="n">
-        <v>0.2261</v>
+        <v>0.2283</v>
       </c>
       <c r="I113" s="21" t="inlineStr">
         <is>
@@ -17572,7 +17572,7 @@
         </is>
       </c>
       <c r="H114" s="29" t="n">
-        <v>0.1503</v>
+        <v>0.1491</v>
       </c>
       <c r="I114" s="27" t="inlineStr">
         <is>
@@ -17615,7 +17615,7 @@
         </is>
       </c>
       <c r="H115" s="23" t="n">
-        <v>0.1128</v>
+        <v>0.1105</v>
       </c>
       <c r="I115" s="21" t="inlineStr">
         <is>
@@ -17658,7 +17658,7 @@
         </is>
       </c>
       <c r="H116" s="31" t="n">
-        <v>0.0417</v>
+        <v>0.0418</v>
       </c>
       <c r="I116" s="27" t="inlineStr">
         <is>
@@ -17744,7 +17744,7 @@
         </is>
       </c>
       <c r="H118" s="31" t="n">
-        <v>0.0242</v>
+        <v>0.0248</v>
       </c>
       <c r="I118" s="27" t="inlineStr">
         <is>
@@ -17787,7 +17787,7 @@
         </is>
       </c>
       <c r="H119" s="25" t="n">
-        <v>0.0217</v>
+        <v>0.0213</v>
       </c>
       <c r="I119" s="21" t="inlineStr">
         <is>
@@ -17816,12 +17816,12 @@
       </c>
       <c r="E120" s="26" t="inlineStr">
         <is>
-          <t>3037</t>
+          <t>2303</t>
         </is>
       </c>
       <c r="F120" s="27" t="inlineStr">
         <is>
-          <t>欣興</t>
+          <t>聯電</t>
         </is>
       </c>
       <c r="G120" s="27" t="inlineStr">
@@ -17830,11 +17830,11 @@
         </is>
       </c>
       <c r="H120" s="31" t="n">
-        <v>0.0206</v>
+        <v>0.0199</v>
       </c>
       <c r="I120" s="27" t="inlineStr">
         <is>
-          <t>193,315</t>
+          <t>1,620,000</t>
         </is>
       </c>
     </row>
@@ -17859,12 +17859,12 @@
       </c>
       <c r="E121" s="20" t="inlineStr">
         <is>
-          <t>2303</t>
+          <t>3037</t>
         </is>
       </c>
       <c r="F121" s="21" t="inlineStr">
         <is>
-          <t>聯電</t>
+          <t>欣興</t>
         </is>
       </c>
       <c r="G121" s="21" t="inlineStr">
@@ -17873,11 +17873,11 @@
         </is>
       </c>
       <c r="H121" s="25" t="n">
-        <v>0.0203</v>
+        <v>0.0197</v>
       </c>
       <c r="I121" s="21" t="inlineStr">
         <is>
-          <t>1,620,000</t>
+          <t>193,315</t>
         </is>
       </c>
     </row>
@@ -17916,7 +17916,7 @@
         </is>
       </c>
       <c r="H122" s="31" t="n">
-        <v>0.0195</v>
+        <v>0.0194</v>
       </c>
       <c r="I122" s="27" t="inlineStr">
         <is>
@@ -17963,7 +17963,7 @@
       </c>
       <c r="I123" s="21" t="inlineStr">
         <is>
-          <t>1,276,794</t>
+          <t>1,284,945</t>
         </is>
       </c>
     </row>
@@ -18002,11 +18002,11 @@
         </is>
       </c>
       <c r="H124" s="29" t="n">
-        <v>0.0922</v>
+        <v>0.0924</v>
       </c>
       <c r="I124" s="27" t="inlineStr">
         <is>
-          <t>634,331</t>
+          <t>638,395</t>
         </is>
       </c>
     </row>
@@ -18045,11 +18045,11 @@
         </is>
       </c>
       <c r="H125" s="23" t="n">
-        <v>0.0771</v>
+        <v>0.0765</v>
       </c>
       <c r="I125" s="21" t="inlineStr">
         <is>
-          <t>196,024</t>
+          <t>197,280</t>
         </is>
       </c>
     </row>
@@ -18088,11 +18088,11 @@
         </is>
       </c>
       <c r="H126" s="31" t="n">
-        <v>0.0467</v>
+        <v>0.04650000000000001</v>
       </c>
       <c r="I126" s="27" t="inlineStr">
         <is>
-          <t>199,624</t>
+          <t>200,903</t>
         </is>
       </c>
     </row>
@@ -18131,11 +18131,11 @@
         </is>
       </c>
       <c r="H127" s="25" t="n">
-        <v>0.0457</v>
+        <v>0.04650000000000001</v>
       </c>
       <c r="I127" s="21" t="inlineStr">
         <is>
-          <t>443,954</t>
+          <t>446,798</t>
         </is>
       </c>
     </row>
@@ -18174,11 +18174,11 @@
         </is>
       </c>
       <c r="H128" s="31" t="n">
-        <v>0.0445</v>
+        <v>0.0449</v>
       </c>
       <c r="I128" s="27" t="inlineStr">
         <is>
-          <t>259,478</t>
+          <t>261,140</t>
         </is>
       </c>
     </row>
@@ -18217,11 +18217,11 @@
         </is>
       </c>
       <c r="H129" s="25" t="n">
-        <v>0.0432</v>
+        <v>0.0436</v>
       </c>
       <c r="I129" s="21" t="inlineStr">
         <is>
-          <t>360,152</t>
+          <t>362,459</t>
         </is>
       </c>
     </row>
@@ -18246,12 +18246,12 @@
       </c>
       <c r="E130" s="26" t="inlineStr">
         <is>
-          <t>INTC.US</t>
+          <t>QCOM.US</t>
         </is>
       </c>
       <c r="F130" s="27" t="inlineStr">
         <is>
-          <t>Intel Corp</t>
+          <t>QUALCOMM INC</t>
         </is>
       </c>
       <c r="G130" s="27" t="inlineStr">
@@ -18260,11 +18260,11 @@
         </is>
       </c>
       <c r="H130" s="31" t="n">
-        <v>0.042</v>
+        <v>0.04219999999999999</v>
       </c>
       <c r="I130" s="27" t="inlineStr">
         <is>
-          <t>1,049,796</t>
+          <t>554,724</t>
         </is>
       </c>
     </row>
@@ -18289,12 +18289,12 @@
       </c>
       <c r="E131" s="20" t="inlineStr">
         <is>
-          <t>QCOM.US</t>
+          <t>INTC.US</t>
         </is>
       </c>
       <c r="F131" s="21" t="inlineStr">
         <is>
-          <t>QUALCOMM INC</t>
+          <t>Intel Corp</t>
         </is>
       </c>
       <c r="G131" s="21" t="inlineStr">
@@ -18303,11 +18303,11 @@
         </is>
       </c>
       <c r="H131" s="25" t="n">
-        <v>0.0416</v>
+        <v>0.04190000000000001</v>
       </c>
       <c r="I131" s="21" t="inlineStr">
         <is>
-          <t>551,192</t>
+          <t>1,056,522</t>
         </is>
       </c>
     </row>
@@ -18346,11 +18346,11 @@
         </is>
       </c>
       <c r="H132" s="31" t="n">
-        <v>0.0413</v>
+        <v>0.04190000000000001</v>
       </c>
       <c r="I132" s="27" t="inlineStr">
         <is>
-          <t>226,253</t>
+          <t>227,702</t>
         </is>
       </c>
     </row>
@@ -18375,12 +18375,12 @@
       </c>
       <c r="E133" s="20" t="inlineStr">
         <is>
-          <t>AAPL.US</t>
+          <t>MSFT.US</t>
         </is>
       </c>
       <c r="F133" s="21" t="inlineStr">
         <is>
-          <t>Apple Inc.</t>
+          <t>Microsoft Corp</t>
         </is>
       </c>
       <c r="G133" s="21" t="inlineStr">
@@ -18389,11 +18389,11 @@
         </is>
       </c>
       <c r="H133" s="23" t="n">
-        <v>0.092</v>
+        <v>0.09179999999999999</v>
       </c>
       <c r="I133" s="21" t="inlineStr">
         <is>
-          <t>50,599</t>
+          <t>32,454</t>
         </is>
       </c>
     </row>
@@ -18418,12 +18418,12 @@
       </c>
       <c r="E134" s="26" t="inlineStr">
         <is>
-          <t>MSFT.US</t>
+          <t>AAPL.US</t>
         </is>
       </c>
       <c r="F134" s="27" t="inlineStr">
         <is>
-          <t>Microsoft Corp</t>
+          <t>Apple Inc.</t>
         </is>
       </c>
       <c r="G134" s="27" t="inlineStr">
@@ -18432,11 +18432,11 @@
         </is>
       </c>
       <c r="H134" s="29" t="n">
-        <v>0.09179999999999999</v>
+        <v>0.09130000000000001</v>
       </c>
       <c r="I134" s="27" t="inlineStr">
         <is>
-          <t>32,454</t>
+          <t>50,599</t>
         </is>
       </c>
     </row>
@@ -18518,7 +18518,7 @@
         </is>
       </c>
       <c r="H136" s="29" t="n">
-        <v>0.0702</v>
+        <v>0.0703</v>
       </c>
       <c r="I136" s="27" t="inlineStr">
         <is>
@@ -18561,7 +18561,7 @@
         </is>
       </c>
       <c r="H137" s="25" t="n">
-        <v>0.0488</v>
+        <v>0.0484</v>
       </c>
       <c r="I137" s="21" t="inlineStr">
         <is>
@@ -18604,7 +18604,7 @@
         </is>
       </c>
       <c r="H138" s="31" t="n">
-        <v>0.0483</v>
+        <v>0.04769999999999999</v>
       </c>
       <c r="I138" s="27" t="inlineStr">
         <is>
@@ -18647,7 +18647,7 @@
         </is>
       </c>
       <c r="H139" s="25" t="n">
-        <v>0.0408</v>
+        <v>0.0407</v>
       </c>
       <c r="I139" s="21" t="inlineStr">
         <is>
@@ -18690,7 +18690,7 @@
         </is>
       </c>
       <c r="H140" s="31" t="n">
-        <v>0.0394</v>
+        <v>0.0392</v>
       </c>
       <c r="I140" s="27" t="inlineStr">
         <is>
@@ -18733,7 +18733,7 @@
         </is>
       </c>
       <c r="H141" s="25" t="n">
-        <v>0.0391</v>
+        <v>0.0387</v>
       </c>
       <c r="I141" s="21" t="inlineStr">
         <is>
@@ -18776,7 +18776,7 @@
         </is>
       </c>
       <c r="H142" s="31" t="n">
-        <v>0.0213</v>
+        <v>0.0212</v>
       </c>
       <c r="I142" s="27" t="inlineStr">
         <is>
@@ -18819,7 +18819,7 @@
         </is>
       </c>
       <c r="H143" s="23" t="n">
-        <v>0.2597</v>
+        <v>0.2596</v>
       </c>
       <c r="I143" s="21" t="inlineStr">
         <is>
@@ -18862,7 +18862,7 @@
         </is>
       </c>
       <c r="H144" s="29" t="n">
-        <v>0.1443</v>
+        <v>0.1447</v>
       </c>
       <c r="I144" s="27" t="inlineStr">
         <is>
@@ -18905,7 +18905,7 @@
         </is>
       </c>
       <c r="H145" s="23" t="n">
-        <v>0.1232</v>
+        <v>0.1258</v>
       </c>
       <c r="I145" s="21" t="inlineStr">
         <is>
@@ -18948,11 +18948,11 @@
         </is>
       </c>
       <c r="H146" s="29" t="n">
-        <v>0.1016</v>
+        <v>0.1034</v>
       </c>
       <c r="I146" s="27" t="inlineStr">
         <is>
-          <t>173,470</t>
+          <t>174,470</t>
         </is>
       </c>
     </row>
@@ -18991,11 +18991,11 @@
         </is>
       </c>
       <c r="H147" s="23" t="n">
-        <v>0.0549</v>
+        <v>0.0528</v>
       </c>
       <c r="I147" s="21" t="inlineStr">
         <is>
-          <t>285,200</t>
+          <t>288,032</t>
         </is>
       </c>
     </row>
@@ -19034,11 +19034,11 @@
         </is>
       </c>
       <c r="H148" s="31" t="n">
-        <v>0.04</v>
+        <v>0.0392</v>
       </c>
       <c r="I148" s="27" t="inlineStr">
         <is>
-          <t>471,800</t>
+          <t>474,100</t>
         </is>
       </c>
     </row>
@@ -19063,25 +19063,25 @@
       </c>
       <c r="E149" s="20" t="inlineStr">
         <is>
-          <t>EMR.US</t>
+          <t>2308</t>
         </is>
       </c>
       <c r="F149" s="21" t="inlineStr">
         <is>
-          <t>Emerson Electric Co</t>
+          <t>台達電</t>
         </is>
       </c>
       <c r="G149" s="21" t="inlineStr">
         <is>
-          <t>海外/全球股票</t>
+          <t>科技電子</t>
         </is>
       </c>
       <c r="H149" s="25" t="n">
-        <v>0.0375</v>
+        <v>0.0335</v>
       </c>
       <c r="I149" s="21" t="inlineStr">
         <is>
-          <t>110,214</t>
+          <t>319,000</t>
         </is>
       </c>
     </row>
@@ -19106,25 +19106,25 @@
       </c>
       <c r="E150" s="26" t="inlineStr">
         <is>
-          <t>2308</t>
+          <t>IFX.GR</t>
         </is>
       </c>
       <c r="F150" s="27" t="inlineStr">
         <is>
-          <t>台達電</t>
+          <t>Infineon Technolo N</t>
         </is>
       </c>
       <c r="G150" s="27" t="inlineStr">
         <is>
-          <t>科技電子</t>
+          <t>其他產業</t>
         </is>
       </c>
       <c r="H150" s="31" t="n">
-        <v>0.0341</v>
+        <v>0.0276</v>
       </c>
       <c r="I150" s="27" t="inlineStr">
         <is>
-          <t>319,000</t>
+          <t>221,786</t>
         </is>
       </c>
     </row>
@@ -19149,25 +19149,25 @@
       </c>
       <c r="E151" s="20" t="inlineStr">
         <is>
-          <t>IFX.GR</t>
+          <t>NXPI.US</t>
         </is>
       </c>
       <c r="F151" s="21" t="inlineStr">
         <is>
-          <t>Infineon Technolo N</t>
+          <t>NXP SEMICONDUCTORS</t>
         </is>
       </c>
       <c r="G151" s="21" t="inlineStr">
         <is>
-          <t>其他產業</t>
+          <t>海外/全球股票</t>
         </is>
       </c>
       <c r="H151" s="25" t="n">
-        <v>0.0269</v>
+        <v>0.0256</v>
       </c>
       <c r="I151" s="21" t="inlineStr">
         <is>
-          <t>217,261</t>
+          <t>50,526</t>
         </is>
       </c>
     </row>
@@ -19206,11 +19206,11 @@
         </is>
       </c>
       <c r="H152" s="31" t="n">
-        <v>0.0251</v>
+        <v>0.0248</v>
       </c>
       <c r="I152" s="27" t="inlineStr">
         <is>
-          <t>469,200</t>
+          <t>474,000</t>
         </is>
       </c>
     </row>
@@ -23639,7 +23639,7 @@
         </is>
       </c>
       <c r="F2" s="43" t="n">
-        <v>103.45</v>
+        <v>105.75</v>
       </c>
       <c r="G2" s="44" t="n">
         <v>0.00911528</v>
@@ -23697,7 +23697,7 @@
         </is>
       </c>
       <c r="F3" s="47" t="n">
-        <v>96</v>
+        <v>98.2</v>
       </c>
       <c r="G3" s="48" t="n">
         <v>-0.04014465</v>
@@ -23755,7 +23755,7 @@
         </is>
       </c>
       <c r="F4" s="43" t="n">
-        <v>115.17</v>
+        <v>115.27</v>
       </c>
       <c r="G4" s="44" t="n">
         <v>0.00866128</v>
@@ -23813,7 +23813,7 @@
         </is>
       </c>
       <c r="F5" s="47" t="n">
-        <v>84.95999999999999</v>
+        <v>84.83</v>
       </c>
       <c r="G5" s="49" t="n">
         <v>0.06664248</v>
@@ -23871,7 +23871,7 @@
         </is>
       </c>
       <c r="F6" s="43" t="n">
-        <v>56.22</v>
+        <v>56.13</v>
       </c>
       <c r="G6" s="44" t="n">
         <v>0.06641135000000001</v>
@@ -23929,7 +23929,7 @@
         </is>
       </c>
       <c r="F7" s="47" t="n">
-        <v>350.57</v>
+        <v>351.88</v>
       </c>
       <c r="G7" s="49" t="n">
         <v>0.04333726</v>
@@ -23987,7 +23987,7 @@
         </is>
       </c>
       <c r="F8" s="43" t="n">
-        <v>49.11</v>
+        <v>49.55</v>
       </c>
       <c r="G8" s="44" t="n">
         <v>0.04219119</v>
@@ -24045,7 +24045,7 @@
         </is>
       </c>
       <c r="F9" s="47" t="n">
-        <v>81</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="G9" s="48" t="n">
         <v>-0.11655405</v>
@@ -24103,7 +24103,7 @@
         </is>
       </c>
       <c r="F10" s="43" t="n">
-        <v>174.47</v>
+        <v>174.31</v>
       </c>
       <c r="G10" s="50" t="n">
         <v>-0.04380673</v>
@@ -24161,7 +24161,7 @@
         </is>
       </c>
       <c r="F11" s="47" t="n">
-        <v>39.56</v>
+        <v>39.98</v>
       </c>
       <c r="G11" s="49" t="n">
         <v>0.05804878</v>
@@ -24219,7 +24219,7 @@
         </is>
       </c>
       <c r="F12" s="43" t="n">
-        <v>34.88</v>
+        <v>35.39</v>
       </c>
       <c r="G12" s="44" t="n">
         <v>0.07029505</v>
@@ -24277,7 +24277,7 @@
         </is>
       </c>
       <c r="F13" s="47" t="n">
-        <v>43.4</v>
+        <v>44</v>
       </c>
       <c r="G13" s="48" t="n">
         <v>-0.04295893000000001</v>
@@ -24335,7 +24335,7 @@
         </is>
       </c>
       <c r="F14" s="43" t="n">
-        <v>63.7</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="G14" s="44" t="n">
         <v>0.03063547</v>
@@ -24393,7 +24393,7 @@
         </is>
       </c>
       <c r="F15" s="47" t="n">
-        <v>27.98</v>
+        <v>27.91</v>
       </c>
       <c r="G15" s="49" t="n">
         <v>0.05632139</v>
@@ -24451,7 +24451,7 @@
         </is>
       </c>
       <c r="F16" s="43" t="n">
-        <v>9.780799999999999</v>
+        <v>9.849600000000001</v>
       </c>
       <c r="G16" s="50" t="n">
         <v>-0.02358716</v>
@@ -24509,7 +24509,7 @@
         </is>
       </c>
       <c r="F17" s="47" t="n">
-        <v>9.790900000000001</v>
+        <v>9.8598</v>
       </c>
       <c r="G17" s="48" t="n">
         <v>-0.02359118</v>
@@ -24567,7 +24567,7 @@
         </is>
       </c>
       <c r="F18" s="43" t="n">
-        <v>25.76</v>
+        <v>25.63</v>
       </c>
       <c r="G18" s="50" t="n">
         <v>-0.09624573</v>
@@ -24625,7 +24625,7 @@
         </is>
       </c>
       <c r="F19" s="47" t="n">
-        <v>7.9194</v>
+        <v>7.9501</v>
       </c>
       <c r="G19" s="48" t="n">
         <v>-0.01325601</v>
@@ -24683,7 +24683,7 @@
         </is>
       </c>
       <c r="F20" s="43" t="n">
-        <v>7.8925</v>
+        <v>7.9231</v>
       </c>
       <c r="G20" s="50" t="n">
         <v>-0.01326918</v>
@@ -24741,7 +24741,7 @@
         </is>
       </c>
       <c r="F21" s="47" t="n">
-        <v>8.444000000000001</v>
+        <v>8.4801</v>
       </c>
       <c r="G21" s="48" t="n">
         <v>-0.04286634</v>
@@ -24799,7 +24799,7 @@
         </is>
       </c>
       <c r="F22" s="43" t="n">
-        <v>8.441599999999999</v>
+        <v>8.4778</v>
       </c>
       <c r="G22" s="50" t="n">
         <v>-0.04286672</v>
@@ -24857,7 +24857,7 @@
         </is>
       </c>
       <c r="F23" s="47" t="n">
-        <v>15.4</v>
+        <v>15.36</v>
       </c>
       <c r="G23" s="48" t="n">
         <v>-0.07210569999999999</v>
@@ -24915,7 +24915,7 @@
         </is>
       </c>
       <c r="F24" s="43" t="n">
-        <v>33.42</v>
+        <v>33.39</v>
       </c>
       <c r="G24" s="50" t="n">
         <v>-0.07485287</v>
@@ -24973,7 +24973,7 @@
         </is>
       </c>
       <c r="F25" s="47" t="n">
-        <v>14.61</v>
+        <v>14.84</v>
       </c>
       <c r="G25" s="51" t="inlineStr"/>
       <c r="H25" s="51" t="inlineStr"/>
@@ -25146,18 +25146,18 @@
         </is>
       </c>
       <c r="F2" s="43" t="n">
-        <v>14.61</v>
+        <v>14.84</v>
       </c>
       <c r="G2" s="41" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="H2" s="52" t="n">
-        <v>-0.24</v>
-      </c>
-      <c r="I2" s="50" t="n">
-        <v>-0.0162</v>
+        <v>0.23</v>
+      </c>
+      <c r="I2" s="44" t="n">
+        <v>0.0157</v>
       </c>
       <c r="J2" s="53" t="inlineStr"/>
       <c r="K2" s="53" t="inlineStr"/>
@@ -25208,18 +25208,18 @@
         </is>
       </c>
       <c r="F3" s="47" t="n">
-        <v>34.88</v>
+        <v>35.39</v>
       </c>
       <c r="G3" s="45" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="H3" s="54" t="n">
-        <v>4.88</v>
+        <v>0.51</v>
       </c>
       <c r="I3" s="49" t="n">
-        <v>0.1627</v>
+        <v>0.0146</v>
       </c>
       <c r="J3" s="49" t="n">
         <v>0.07029505</v>
@@ -25282,18 +25282,18 @@
         </is>
       </c>
       <c r="F4" s="43" t="n">
-        <v>15.4</v>
+        <v>15.36</v>
       </c>
       <c r="G4" s="41" t="inlineStr">
         <is>
-          <t>10/20</t>
-        </is>
-      </c>
-      <c r="H4" s="52" t="n">
-        <v>-0.03</v>
+          <t>10/21</t>
+        </is>
+      </c>
+      <c r="H4" s="55" t="n">
+        <v>-0.04</v>
       </c>
       <c r="I4" s="50" t="n">
-        <v>-0.0019</v>
+        <v>-0.0026</v>
       </c>
       <c r="J4" s="50" t="n">
         <v>-0.07210569999999999</v>
@@ -25356,18 +25356,18 @@
         </is>
       </c>
       <c r="F5" s="47" t="n">
-        <v>33.42</v>
+        <v>33.39</v>
       </c>
       <c r="G5" s="45" t="inlineStr">
         <is>
-          <t>10/20</t>
-        </is>
-      </c>
-      <c r="H5" s="55" t="n">
-        <v>-0.19</v>
+          <t>10/21</t>
+        </is>
+      </c>
+      <c r="H5" s="56" t="n">
+        <v>-0.03</v>
       </c>
       <c r="I5" s="48" t="n">
-        <v>-0.005699999999999999</v>
+        <v>-0.0009</v>
       </c>
       <c r="J5" s="48" t="n">
         <v>-0.07485287</v>
@@ -25430,18 +25430,18 @@
         </is>
       </c>
       <c r="F6" s="43" t="n">
-        <v>49.11</v>
+        <v>49.55</v>
       </c>
       <c r="G6" s="41" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="H6" s="52" t="n">
-        <v>-4.04</v>
-      </c>
-      <c r="I6" s="50" t="n">
-        <v>-0.076</v>
+        <v>0.44</v>
+      </c>
+      <c r="I6" s="44" t="n">
+        <v>0.009000000000000001</v>
       </c>
       <c r="J6" s="44" t="n">
         <v>0.04219119</v>
@@ -25500,18 +25500,18 @@
         </is>
       </c>
       <c r="F7" s="47" t="n">
-        <v>39.56</v>
+        <v>39.98</v>
       </c>
       <c r="G7" s="45" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="H7" s="54" t="n">
-        <v>1.23</v>
+        <v>0.42</v>
       </c>
       <c r="I7" s="49" t="n">
-        <v>0.0321</v>
+        <v>0.0106</v>
       </c>
       <c r="J7" s="49" t="n">
         <v>0.05804878</v>
@@ -25574,18 +25574,18 @@
         </is>
       </c>
       <c r="F8" s="43" t="n">
-        <v>103.45</v>
+        <v>105.75</v>
       </c>
       <c r="G8" s="41" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="H8" s="52" t="n">
-        <v>-1.95</v>
-      </c>
-      <c r="I8" s="50" t="n">
-        <v>-0.0185</v>
+        <v>2.3</v>
+      </c>
+      <c r="I8" s="44" t="n">
+        <v>0.0222</v>
       </c>
       <c r="J8" s="44" t="n">
         <v>0.00911528</v>
@@ -25644,18 +25644,18 @@
         </is>
       </c>
       <c r="F9" s="47" t="n">
-        <v>27.98</v>
+        <v>27.91</v>
       </c>
       <c r="G9" s="45" t="inlineStr">
         <is>
-          <t>10/20</t>
-        </is>
-      </c>
-      <c r="H9" s="55" t="n">
-        <v>-0.04</v>
+          <t>10/21</t>
+        </is>
+      </c>
+      <c r="H9" s="56" t="n">
+        <v>-0.07000000000000001</v>
       </c>
       <c r="I9" s="48" t="n">
-        <v>-0.0014</v>
+        <v>-0.0025</v>
       </c>
       <c r="J9" s="49" t="n">
         <v>0.05632139</v>
@@ -25718,18 +25718,18 @@
         </is>
       </c>
       <c r="F10" s="43" t="n">
-        <v>25.76</v>
+        <v>25.63</v>
       </c>
       <c r="G10" s="41" t="inlineStr">
         <is>
-          <t>10/20</t>
-        </is>
-      </c>
-      <c r="H10" s="52" t="n">
-        <v>-2.8</v>
+          <t>10/21</t>
+        </is>
+      </c>
+      <c r="H10" s="55" t="n">
+        <v>-0.13</v>
       </c>
       <c r="I10" s="50" t="n">
-        <v>-0.098</v>
+        <v>-0.005</v>
       </c>
       <c r="J10" s="50" t="n">
         <v>-0.09624573</v>
@@ -25788,18 +25788,18 @@
         </is>
       </c>
       <c r="F11" s="47" t="n">
-        <v>49.11</v>
+        <v>49.55</v>
       </c>
       <c r="G11" s="45" t="inlineStr">
         <is>
-          <t>10/20</t>
-        </is>
-      </c>
-      <c r="H11" s="55" t="n">
-        <v>-4.04</v>
-      </c>
-      <c r="I11" s="48" t="n">
-        <v>-0.076</v>
+          <t>10/21</t>
+        </is>
+      </c>
+      <c r="H11" s="54" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="I11" s="49" t="n">
+        <v>0.009000000000000001</v>
       </c>
       <c r="J11" s="49" t="n">
         <v>0.04219119</v>
@@ -25858,18 +25858,18 @@
         </is>
       </c>
       <c r="F12" s="43" t="n">
-        <v>96</v>
+        <v>98.2</v>
       </c>
       <c r="G12" s="41" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="H12" s="52" t="n">
-        <v>-12.3</v>
-      </c>
-      <c r="I12" s="50" t="n">
-        <v>-0.1136</v>
+        <v>2.2</v>
+      </c>
+      <c r="I12" s="44" t="n">
+        <v>0.0229</v>
       </c>
       <c r="J12" s="50" t="n">
         <v>-0.04014465</v>
@@ -25928,18 +25928,18 @@
         </is>
       </c>
       <c r="F13" s="47" t="n">
-        <v>81</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="G13" s="45" t="inlineStr">
         <is>
-          <t>10/20</t>
-        </is>
-      </c>
-      <c r="H13" s="55" t="n">
-        <v>-6.5</v>
-      </c>
-      <c r="I13" s="48" t="n">
-        <v>-0.07429999999999999</v>
+          <t>10/21</t>
+        </is>
+      </c>
+      <c r="H13" s="54" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="I13" s="49" t="n">
+        <v>0.0198</v>
       </c>
       <c r="J13" s="48" t="n">
         <v>-0.11655405</v>
@@ -25998,18 +25998,18 @@
         </is>
       </c>
       <c r="F14" s="43" t="n">
-        <v>63.7</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="G14" s="41" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="H14" s="52" t="n">
-        <v>-2.5</v>
-      </c>
-      <c r="I14" s="50" t="n">
-        <v>-0.0378</v>
+        <v>0.4</v>
+      </c>
+      <c r="I14" s="44" t="n">
+        <v>0.0063</v>
       </c>
       <c r="J14" s="44" t="n">
         <v>0.03063547</v>
@@ -26068,18 +26068,18 @@
         </is>
       </c>
       <c r="F15" s="47" t="n">
-        <v>43.4</v>
+        <v>44</v>
       </c>
       <c r="G15" s="45" t="inlineStr">
         <is>
-          <t>10/20</t>
-        </is>
-      </c>
-      <c r="H15" s="55" t="n">
-        <v>-3.2</v>
-      </c>
-      <c r="I15" s="48" t="n">
-        <v>-0.0687</v>
+          <t>10/21</t>
+        </is>
+      </c>
+      <c r="H15" s="54" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I15" s="49" t="n">
+        <v>0.0138</v>
       </c>
       <c r="J15" s="48" t="n">
         <v>-0.04295893000000001</v>
@@ -26138,18 +26138,18 @@
         </is>
       </c>
       <c r="F16" s="43" t="n">
-        <v>14.61</v>
+        <v>14.84</v>
       </c>
       <c r="G16" s="41" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="H16" s="52" t="n">
-        <v>-0.24</v>
-      </c>
-      <c r="I16" s="50" t="n">
-        <v>-0.0162</v>
+        <v>0.23</v>
+      </c>
+      <c r="I16" s="44" t="n">
+        <v>0.0157</v>
       </c>
       <c r="J16" s="53" t="inlineStr"/>
       <c r="K16" s="53" t="inlineStr"/>
@@ -26328,18 +26328,18 @@
         </is>
       </c>
       <c r="F2" s="43" t="n">
-        <v>56.22</v>
+        <v>56.13</v>
       </c>
       <c r="G2" s="43" t="inlineStr">
         <is>
-          <t>10/19</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="H2" s="52" t="n">
-        <v>-0.44</v>
-      </c>
-      <c r="I2" s="50" t="n">
-        <v>-0.007800000000000001</v>
+        <v>0.97</v>
+      </c>
+      <c r="I2" s="44" t="n">
+        <v>0.0176</v>
       </c>
       <c r="J2" s="44" t="n">
         <v>0.06641135000000001</v>
@@ -26402,18 +26402,18 @@
         </is>
       </c>
       <c r="F3" s="47" t="n">
-        <v>9.790900000000001</v>
+        <v>9.8598</v>
       </c>
       <c r="G3" s="47" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H3" s="55" t="n">
-        <v>-0.0844</v>
-      </c>
-      <c r="I3" s="48" t="n">
-        <v>-0.008500000000000001</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H3" s="54" t="n">
+        <v>0.0323</v>
+      </c>
+      <c r="I3" s="49" t="n">
+        <v>0.0033</v>
       </c>
       <c r="J3" s="48" t="n">
         <v>-0.02359118</v>
@@ -26476,18 +26476,18 @@
         </is>
       </c>
       <c r="F4" s="43" t="n">
-        <v>7.8925</v>
+        <v>7.9231</v>
       </c>
       <c r="G4" s="43" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H4" s="56" t="n">
-        <v>0.0009</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H4" s="52" t="n">
+        <v>0.014</v>
       </c>
       <c r="I4" s="44" t="n">
-        <v>0.0001</v>
+        <v>0.0018</v>
       </c>
       <c r="J4" s="50" t="n">
         <v>-0.01326918</v>
@@ -26550,18 +26550,18 @@
         </is>
       </c>
       <c r="F5" s="47" t="n">
-        <v>8.444000000000001</v>
+        <v>8.4801</v>
       </c>
       <c r="G5" s="47" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H5" s="55" t="n">
-        <v>-0.0069</v>
-      </c>
-      <c r="I5" s="48" t="n">
-        <v>-0.0008</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H5" s="54" t="n">
+        <v>0.0474</v>
+      </c>
+      <c r="I5" s="49" t="n">
+        <v>0.005600000000000001</v>
       </c>
       <c r="J5" s="48" t="n">
         <v>-0.04286634</v>
@@ -26624,18 +26624,18 @@
         </is>
       </c>
       <c r="F6" s="43" t="n">
-        <v>9.780799999999999</v>
+        <v>9.849600000000001</v>
       </c>
       <c r="G6" s="43" t="inlineStr">
         <is>
-          <t>10/16</t>
+          <t>10/20</t>
         </is>
       </c>
       <c r="H6" s="52" t="n">
-        <v>-0.0843</v>
-      </c>
-      <c r="I6" s="50" t="n">
-        <v>-0.008500000000000001</v>
+        <v>0.0322</v>
+      </c>
+      <c r="I6" s="44" t="n">
+        <v>0.0033</v>
       </c>
       <c r="J6" s="50" t="n">
         <v>-0.02358716</v>
@@ -26698,18 +26698,18 @@
         </is>
       </c>
       <c r="F7" s="47" t="n">
-        <v>8.441599999999999</v>
+        <v>8.4778</v>
       </c>
       <c r="G7" s="47" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H7" s="55" t="n">
-        <v>-0.007</v>
-      </c>
-      <c r="I7" s="48" t="n">
-        <v>-0.0008</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H7" s="54" t="n">
+        <v>0.0474</v>
+      </c>
+      <c r="I7" s="49" t="n">
+        <v>0.005600000000000001</v>
       </c>
       <c r="J7" s="48" t="n">
         <v>-0.04286672</v>
@@ -26772,18 +26772,18 @@
         </is>
       </c>
       <c r="F8" s="43" t="n">
-        <v>7.9194</v>
+        <v>7.9501</v>
       </c>
       <c r="G8" s="43" t="inlineStr">
         <is>
-          <t>10/16</t>
-        </is>
-      </c>
-      <c r="H8" s="56" t="n">
-        <v>0.0009</v>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="H8" s="52" t="n">
+        <v>0.014</v>
       </c>
       <c r="I8" s="44" t="n">
-        <v>0.0001</v>
+        <v>0.0018</v>
       </c>
       <c r="J8" s="50" t="n">
         <v>-0.01325601</v>
@@ -26846,18 +26846,18 @@
         </is>
       </c>
       <c r="F9" s="47" t="n">
-        <v>84.95999999999999</v>
+        <v>84.83</v>
       </c>
       <c r="G9" s="47" t="inlineStr">
         <is>
-          <t>10/19</t>
-        </is>
-      </c>
-      <c r="H9" s="55" t="n">
-        <v>-0.66</v>
-      </c>
-      <c r="I9" s="48" t="n">
-        <v>-0.0077</v>
+          <t>10/21</t>
+        </is>
+      </c>
+      <c r="H9" s="54" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="I9" s="49" t="n">
+        <v>0.0178</v>
       </c>
       <c r="J9" s="49" t="n">
         <v>0.06664248</v>
@@ -26920,18 +26920,18 @@
         </is>
       </c>
       <c r="F10" s="43" t="n">
-        <v>174.47</v>
+        <v>174.31</v>
       </c>
       <c r="G10" s="43" t="inlineStr">
         <is>
-          <t>10/19</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="H10" s="52" t="n">
-        <v>-1.11</v>
-      </c>
-      <c r="I10" s="50" t="n">
-        <v>-0.0063</v>
+        <v>4.47</v>
+      </c>
+      <c r="I10" s="44" t="n">
+        <v>0.0263</v>
       </c>
       <c r="J10" s="50" t="n">
         <v>-0.04380673</v>
@@ -26994,18 +26994,18 @@
         </is>
       </c>
       <c r="F11" s="47" t="n">
-        <v>115.17</v>
+        <v>115.27</v>
       </c>
       <c r="G11" s="47" t="inlineStr">
         <is>
-          <t>10/19</t>
-        </is>
-      </c>
-      <c r="H11" s="55" t="n">
-        <v>-0.85</v>
-      </c>
-      <c r="I11" s="48" t="n">
-        <v>-0.0073</v>
+          <t>10/21</t>
+        </is>
+      </c>
+      <c r="H11" s="54" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="I11" s="49" t="n">
+        <v>0.0254</v>
       </c>
       <c r="J11" s="49" t="n">
         <v>0.00866128</v>
@@ -27064,18 +27064,18 @@
         </is>
       </c>
       <c r="F12" s="43" t="n">
-        <v>350.57</v>
+        <v>351.88</v>
       </c>
       <c r="G12" s="43" t="inlineStr">
         <is>
-          <t>10/19</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="H12" s="52" t="n">
-        <v>-2.41</v>
-      </c>
-      <c r="I12" s="50" t="n">
-        <v>-0.0068</v>
+        <v>10.4</v>
+      </c>
+      <c r="I12" s="44" t="n">
+        <v>0.0305</v>
       </c>
       <c r="J12" s="44" t="n">
         <v>0.04333726</v>

</xml_diff>